<commit_message>
auto: reporte semana 2026-08-03 → 2026-08-09
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,36 +420,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B2">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/07/27 13:34:48</v>
+        <v>2026/08/04 00:14:07</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/07/27 14:00:34</v>
+        <v>2026/08/04 00:22:16</v>
       </c>
       <c r="E2" t="str">
-        <v>00:25:46</v>
+        <v>00:08:09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B3">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/07/27 14:39:09</v>
+        <v>2026/08/07 20:58:11</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/07/27 15:56:16</v>
+        <v>2026/08/07 21:08:52</v>
       </c>
       <c r="E3" t="str">
-        <v>01:17:07</v>
+        <v>00:10:41</v>
       </c>
     </row>
     <row r="4">
@@ -460,13 +460,13 @@
         <v>3841</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/07/27 17:30:08</v>
+        <v>2026/08/03 14:59:28</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/07/27 17:31:54</v>
+        <v>2026/08/03 15:13:24</v>
       </c>
       <c r="E4" t="str">
-        <v>00:01:46</v>
+        <v>00:13:56</v>
       </c>
     </row>
     <row r="5">
@@ -477,13 +477,13 @@
         <v>3841</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/07/27 18:32:36</v>
+        <v>2026/08/03 15:23:32</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/07/27 18:35:51</v>
+        <v>2026/08/03 15:42:50</v>
       </c>
       <c r="E5" t="str">
-        <v>00:03:15</v>
+        <v>00:19:18</v>
       </c>
     </row>
     <row r="6">
@@ -494,13 +494,13 @@
         <v>3841</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/07/27 19:32:55</v>
+        <v>2026/08/03 17:37:48</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/07/27 20:22:58</v>
+        <v>2026/08/03 18:53:32</v>
       </c>
       <c r="E6" t="str">
-        <v>00:50:03</v>
+        <v>01:15:44</v>
       </c>
     </row>
     <row r="7">
@@ -511,13 +511,13 @@
         <v>3841</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/07/27 20:45:58</v>
+        <v>2026/08/03 22:30:15</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/07/27 21:10:14</v>
+        <v>2026/08/03 22:31:24</v>
       </c>
       <c r="E7" t="str">
-        <v>00:24:16</v>
+        <v>00:01:09</v>
       </c>
     </row>
     <row r="8">
@@ -528,13 +528,13 @@
         <v>3841</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/07/27 21:50:35</v>
+        <v>2026/08/04 16:06:38</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/07/27 22:08:20</v>
+        <v>2026/08/04 16:10:55</v>
       </c>
       <c r="E8" t="str">
-        <v>00:17:45</v>
+        <v>00:04:17</v>
       </c>
     </row>
     <row r="9">
@@ -545,13 +545,13 @@
         <v>3841</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/07/27 22:23:35</v>
+        <v>2026/08/04 16:38:16</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/07/27 22:36:39</v>
+        <v>2026/08/04 16:49:22</v>
       </c>
       <c r="E9" t="str">
-        <v>00:13:04</v>
+        <v>00:11:06</v>
       </c>
     </row>
     <row r="10">
@@ -562,13 +562,13 @@
         <v>3841</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/07/28 02:34:49</v>
+        <v>2026/08/04 18:22:28</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/07/28 02:44:51</v>
+        <v>2026/08/04 18:27:40</v>
       </c>
       <c r="E10" t="str">
-        <v>00:10:02</v>
+        <v>00:05:12</v>
       </c>
     </row>
     <row r="11">
@@ -579,13 +579,13 @@
         <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/07/28 13:21:06</v>
+        <v>2026/08/04 20:15:29</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/07/28 14:04:05</v>
+        <v>2026/08/04 20:26:49</v>
       </c>
       <c r="E11" t="str">
-        <v>00:42:59</v>
+        <v>00:11:20</v>
       </c>
     </row>
     <row r="12">
@@ -596,13 +596,13 @@
         <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/07/28 14:35:30</v>
+        <v>2026/08/05 13:09:08</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/07/28 14:49:15</v>
+        <v>2026/08/05 13:26:56</v>
       </c>
       <c r="E12" t="str">
-        <v>00:13:45</v>
+        <v>00:17:48</v>
       </c>
     </row>
     <row r="13">
@@ -613,13 +613,13 @@
         <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/07/28 16:39:55</v>
+        <v>2026/08/05 15:09:54</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/07/28 16:41:47</v>
+        <v>2026/08/05 15:17:45</v>
       </c>
       <c r="E13" t="str">
-        <v>00:01:52</v>
+        <v>00:07:51</v>
       </c>
     </row>
     <row r="14">
@@ -630,13 +630,13 @@
         <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/07/28 19:54:31</v>
+        <v>2026/08/05 16:43:16</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/07/28 20:24:31</v>
+        <v>2026/08/05 16:53:46</v>
       </c>
       <c r="E14" t="str">
-        <v>00:30:00</v>
+        <v>00:10:30</v>
       </c>
     </row>
     <row r="15">
@@ -647,13 +647,13 @@
         <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/07/29 13:28:36</v>
+        <v>2026/08/05 17:15:16</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/07/29 13:55:48</v>
+        <v>2026/08/05 17:22:48</v>
       </c>
       <c r="E15" t="str">
-        <v>00:27:12</v>
+        <v>00:07:32</v>
       </c>
     </row>
     <row r="16">
@@ -664,13 +664,13 @@
         <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/07/29 15:08:07</v>
+        <v>2026/08/06 13:20:04</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/07/29 15:15:09</v>
+        <v>2026/08/06 13:23:50</v>
       </c>
       <c r="E16" t="str">
-        <v>00:07:02</v>
+        <v>00:03:46</v>
       </c>
     </row>
     <row r="17">
@@ -681,13 +681,13 @@
         <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/07/29 16:42:48</v>
+        <v>2026/08/06 18:06:47</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/07/29 17:12:15</v>
+        <v>2026/08/06 18:08:25</v>
       </c>
       <c r="E17" t="str">
-        <v>00:29:27</v>
+        <v>00:01:38</v>
       </c>
     </row>
     <row r="18">
@@ -698,13 +698,13 @@
         <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/07/29 17:39:15</v>
+        <v>2026/08/06 18:24:32</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/07/29 17:45:25</v>
+        <v>2026/08/06 18:48:03</v>
       </c>
       <c r="E18" t="str">
-        <v>00:06:10</v>
+        <v>00:23:31</v>
       </c>
     </row>
     <row r="19">
@@ -715,13 +715,13 @@
         <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/07/29 18:53:31</v>
+        <v>2026/08/06 20:39:05</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/07/29 19:58:45</v>
+        <v>2026/08/06 20:45:39</v>
       </c>
       <c r="E19" t="str">
-        <v>01:05:14</v>
+        <v>00:06:34</v>
       </c>
     </row>
     <row r="20">
@@ -732,13 +732,13 @@
         <v>3841</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/07/30 13:01:09</v>
+        <v>2026/08/07 14:00:31</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/07/30 13:08:44</v>
+        <v>2026/08/07 14:16:16</v>
       </c>
       <c r="E20" t="str">
-        <v>00:07:35</v>
+        <v>00:15:45</v>
       </c>
     </row>
     <row r="21">
@@ -749,13 +749,13 @@
         <v>3841</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/07/30 20:16:41</v>
+        <v>2026/08/07 15:39:36</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/07/30 20:51:01</v>
+        <v>2026/08/07 15:49:20</v>
       </c>
       <c r="E21" t="str">
-        <v>00:34:20</v>
+        <v>00:09:44</v>
       </c>
     </row>
     <row r="22">
@@ -766,13 +766,13 @@
         <v>3841</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/07/31 18:04:58</v>
+        <v>2026/08/07 16:20:55</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/07/31 19:59:09</v>
+        <v>2026/08/07 16:47:51</v>
       </c>
       <c r="E22" t="str">
-        <v>01:54:11</v>
+        <v>00:26:56</v>
       </c>
     </row>
     <row r="23">
@@ -783,13 +783,13 @@
         <v>3841</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/08/01 04:47:28</v>
+        <v>2026/08/07 17:55:13</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/08/01 04:54:37</v>
+        <v>2026/08/07 18:09:50</v>
       </c>
       <c r="E23" t="str">
-        <v>00:07:09</v>
+        <v>00:14:37</v>
       </c>
     </row>
     <row r="24">
@@ -800,47 +800,47 @@
         <v>3841</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/08/02 17:18:31</v>
+        <v>2026/08/07 19:25:23</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/08/02 17:19:53</v>
+        <v>2026/08/07 19:45:36</v>
       </c>
       <c r="E24" t="str">
-        <v>00:01:22</v>
+        <v>00:20:13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B25">
-        <v>4936</v>
+        <v>5209</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/07/31 21:15:59</v>
+        <v>2026/08/04 14:05:03</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/07/31 22:11:48</v>
+        <v>2026/08/04 14:15:15</v>
       </c>
       <c r="E25" t="str">
-        <v>00:55:49</v>
+        <v>00:10:12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B26">
-        <v>4936</v>
+        <v>3860</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/07/31 23:34:38</v>
+        <v>2026/08/03 13:08:36</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/07/31 23:37:30</v>
+        <v>2026/08/03 13:48:22</v>
       </c>
       <c r="E26" t="str">
-        <v>00:02:52</v>
+        <v>00:39:46</v>
       </c>
     </row>
     <row r="27">
@@ -851,13 +851,13 @@
         <v>3860</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/07/29 14:19:49</v>
+        <v>2026/08/03 19:48:56</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/07/29 14:20:58</v>
+        <v>2026/08/03 20:05:16</v>
       </c>
       <c r="E27" t="str">
-        <v>00:01:09</v>
+        <v>00:16:20</v>
       </c>
     </row>
     <row r="28">
@@ -868,13 +868,13 @@
         <v>3860</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/07/30 19:44:10</v>
+        <v>2026/08/07 18:24:06</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/07/30 19:57:33</v>
+        <v>2026/08/07 18:25:27</v>
       </c>
       <c r="E28" t="str">
-        <v>00:13:23</v>
+        <v>00:01:21</v>
       </c>
     </row>
     <row r="29">
@@ -885,64 +885,64 @@
         <v>3860</v>
       </c>
       <c r="C29" t="str">
-        <v>2026/07/30 20:16:18</v>
+        <v>2026/08/08 14:57:00</v>
       </c>
       <c r="D29" t="str">
-        <v>2026/07/30 20:29:00</v>
+        <v>2026/08/08 15:11:59</v>
       </c>
       <c r="E29" t="str">
-        <v>00:12:42</v>
+        <v>00:14:59</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B30">
-        <v>3860</v>
+        <v>5651</v>
       </c>
       <c r="C30" t="str">
-        <v>2026/07/31 17:47:49</v>
+        <v>2026/08/04 13:51:17</v>
       </c>
       <c r="D30" t="str">
-        <v>2026/07/31 19:42:43</v>
+        <v>2026/08/04 13:57:15</v>
       </c>
       <c r="E30" t="str">
-        <v>01:54:54</v>
+        <v>00:05:58</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B31">
-        <v>5633</v>
+        <v>5651</v>
       </c>
       <c r="C31" t="str">
-        <v>2026/07/29 13:57:54</v>
+        <v>2026/08/04 19:06:00</v>
       </c>
       <c r="D31" t="str">
-        <v>2026/07/29 16:12:06</v>
+        <v>2026/08/04 19:08:08</v>
       </c>
       <c r="E31" t="str">
-        <v>02:14:12</v>
+        <v>00:02:08</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B32">
-        <v>5633</v>
+        <v>5651</v>
       </c>
       <c r="C32" t="str">
-        <v>2026/07/30 14:07:47</v>
+        <v>2026/08/07 23:24:56</v>
       </c>
       <c r="D32" t="str">
-        <v>2026/07/30 14:16:07</v>
+        <v>2026/08/07 23:37:44</v>
       </c>
       <c r="E32" t="str">
-        <v>00:08:20</v>
+        <v>00:12:48</v>
       </c>
     </row>
     <row r="33">
@@ -953,13 +953,13 @@
         <v>5633</v>
       </c>
       <c r="C33" t="str">
-        <v>2026/07/30 14:26:37</v>
+        <v>2026/08/04 16:52:54</v>
       </c>
       <c r="D33" t="str">
-        <v>2026/07/30 14:38:59</v>
+        <v>2026/08/04 17:03:20</v>
       </c>
       <c r="E33" t="str">
-        <v>00:12:22</v>
+        <v>00:10:26</v>
       </c>
     </row>
     <row r="34">
@@ -970,161 +970,93 @@
         <v>5633</v>
       </c>
       <c r="C34" t="str">
-        <v>2026/07/30 14:51:32</v>
+        <v>2026/08/05 15:30:12</v>
       </c>
       <c r="D34" t="str">
-        <v>2026/07/30 15:03:31</v>
+        <v>2026/08/05 15:31:13</v>
       </c>
       <c r="E34" t="str">
-        <v>00:11:59</v>
+        <v>00:01:01</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B35">
-        <v>5633</v>
+        <v>5220</v>
       </c>
       <c r="C35" t="str">
-        <v>2026/07/30 15:26:05</v>
+        <v>2026/08/06 14:50:16</v>
       </c>
       <c r="D35" t="str">
-        <v>2026/07/30 15:46:27</v>
+        <v>2026/08/06 15:19:34</v>
       </c>
       <c r="E35" t="str">
-        <v>00:20:22</v>
+        <v>00:29:18</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
       </c>
       <c r="B36">
-        <v>5633</v>
+        <v>5245</v>
       </c>
       <c r="C36" t="str">
-        <v>2026/07/30 16:47:03</v>
+        <v>2026/08/07 22:20:38</v>
       </c>
       <c r="D36" t="str">
-        <v>2026/07/30 16:48:52</v>
+        <v>2026/08/07 22:21:39</v>
       </c>
       <c r="E36" t="str">
-        <v>00:01:49</v>
+        <v>00:01:01</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B37">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C37" t="str">
-        <v>2026/07/27 15:46:14</v>
+        <v>2026/08/07 14:03:01</v>
       </c>
       <c r="D37" t="str">
-        <v>2026/07/27 15:50:31</v>
+        <v>2026/08/07 14:11:34</v>
       </c>
       <c r="E37" t="str">
-        <v>00:04:17</v>
+        <v>00:08:33</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B38">
-        <v>5220</v>
+        <v>5223</v>
       </c>
       <c r="C38" t="str">
-        <v>2026/07/28 20:58:54</v>
+        <v>2026/08/04 12:01:53</v>
       </c>
       <c r="D38" t="str">
-        <v>2026/07/28 21:16:43</v>
+        <v>2026/08/04 12:05:28</v>
       </c>
       <c r="E38" t="str">
-        <v>00:17:49</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
-      </c>
-      <c r="B39">
-        <v>5635</v>
-      </c>
-      <c r="C39" t="str">
-        <v>2026/07/28 06:28:24</v>
-      </c>
-      <c r="D39" t="str">
-        <v>2026/07/28 06:41:26</v>
-      </c>
-      <c r="E39" t="str">
-        <v>00:13:02</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B40">
-        <v>5223</v>
-      </c>
-      <c r="C40" t="str">
-        <v>2026/07/30 15:03:49</v>
-      </c>
-      <c r="D40" t="str">
-        <v>2026/07/30 15:09:51</v>
-      </c>
-      <c r="E40" t="str">
-        <v>00:06:02</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B41">
-        <v>5223</v>
-      </c>
-      <c r="C41" t="str">
-        <v>2026/07/30 15:25:24</v>
-      </c>
-      <c r="D41" t="str">
-        <v>2026/07/30 15:55:12</v>
-      </c>
-      <c r="E41" t="str">
-        <v>00:29:48</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B42">
-        <v>5223</v>
-      </c>
-      <c r="C42" t="str">
-        <v>2026/07/30 19:35:42</v>
-      </c>
-      <c r="D42" t="str">
-        <v>2026/07/30 19:41:13</v>
-      </c>
-      <c r="E42" t="str">
-        <v>00:05:31</v>
+        <v>00:03:35</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1142,30 +1074,30 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-07-27</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>03:33:02</v>
+        <v>00:08:09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-07-28</v>
+        <v>2026-08-07</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>01:38:38</v>
+        <v>00:10:41</v>
       </c>
     </row>
     <row r="4">
@@ -1173,13 +1105,13 @@
         <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-07-29</v>
+        <v>2026-08-03</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" t="str">
-        <v>02:15:05</v>
+        <v>01:50:07</v>
       </c>
     </row>
     <row r="5">
@@ -1187,13 +1119,13 @@
         <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" t="str">
-        <v>00:41:55</v>
+        <v>00:31:55</v>
       </c>
     </row>
     <row r="6">
@@ -1201,13 +1133,13 @@
         <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-07-31</v>
+        <v>2026-08-05</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D6" t="str">
-        <v>01:54:11</v>
+        <v>00:43:41</v>
       </c>
     </row>
     <row r="7">
@@ -1215,13 +1147,13 @@
         <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-08-01</v>
+        <v>2026-08-06</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D7" t="str">
-        <v>00:07:09</v>
+        <v>00:35:29</v>
       </c>
     </row>
     <row r="8">
@@ -1229,27 +1161,27 @@
         <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-02</v>
+        <v>2026-08-07</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8" t="str">
-        <v>00:01:22</v>
+        <v>01:27:15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-07-31</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="str">
-        <v>00:58:41</v>
+        <v>00:10:12</v>
       </c>
     </row>
     <row r="10">
@@ -1257,13 +1189,13 @@
         <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-07-29</v>
+        <v>2026-08-03</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="str">
-        <v>00:01:09</v>
+        <v>00:56:06</v>
       </c>
     </row>
     <row r="11">
@@ -1271,13 +1203,13 @@
         <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-07</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="str">
-        <v>00:26:05</v>
+        <v>00:01:21</v>
       </c>
     </row>
     <row r="12">
@@ -1285,109 +1217,137 @@
         <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-07-31</v>
+        <v>2026-08-08</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="str">
-        <v>01:54:54</v>
+        <v>00:14:59</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-07-29</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>02:14:12</v>
+        <v>00:08:06</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-07</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:54:52</v>
+        <v>00:12:48</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-07-27</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="str">
-        <v>00:04:17</v>
+        <v>00:10:26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-07-28</v>
+        <v>2026-08-05</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="str">
-        <v>00:17:49</v>
+        <v>00:01:01</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-07-28</v>
+        <v>2026-08-06</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="str">
-        <v>00:13:02</v>
+        <v>00:29:18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>00:01:01</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>PEUGEOT SRTR-81 (STGO)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>00:08:33</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
-      <c r="B18" t="str">
-        <v>2026-07-30</v>
-      </c>
-      <c r="C18">
-        <v>3</v>
-      </c>
-      <c r="D18" t="str">
-        <v>00:41:21</v>
+      <c r="B20" t="str">
+        <v>2026-08-04</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="str">
+        <v>00:03:35</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1402,84 +1362,117 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B2">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>10:11:22</v>
+        <v>00:18:50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C3" t="str">
-        <v>00:58:41</v>
+        <v>05:08:27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>02:22:08</v>
+        <v>00:10:12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C5" t="str">
-        <v>03:09:04</v>
+        <v>01:12:26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="str">
-        <v>00:22:06</v>
+        <v>00:20:54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="str">
-        <v>00:13:02</v>
+        <v>00:11:27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="str">
+        <v>00:29:18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="str">
+        <v>00:01:01</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PEUGEOT SRTR-81 (STGO)</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>00:08:33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8" t="str">
-        <v>00:41:21</v>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="str">
+        <v>00:03:35</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-08-10 → 2026-08-16
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,13 +426,13 @@
         <v>6771</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/08/04 00:14:07</v>
+        <v>2026/08/10 18:21:12</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/08/04 00:22:16</v>
+        <v>2026/08/10 18:28:25</v>
       </c>
       <c r="E2" t="str">
-        <v>00:08:09</v>
+        <v>00:07:13</v>
       </c>
     </row>
     <row r="3">
@@ -443,620 +443,1045 @@
         <v>6771</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/08/07 20:58:11</v>
+        <v>2026/08/10 20:58:59</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/08/07 21:08:52</v>
+        <v>2026/08/10 21:06:12</v>
       </c>
       <c r="E3" t="str">
-        <v>00:10:41</v>
+        <v>00:07:13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B4">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/08/03 14:59:28</v>
+        <v>2026/08/11 01:51:22</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/08/03 15:13:24</v>
+        <v>2026/08/11 01:59:04</v>
       </c>
       <c r="E4" t="str">
-        <v>00:13:56</v>
+        <v>00:07:42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B5">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/08/03 15:23:32</v>
+        <v>2026/08/11 16:35:58</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/08/03 15:42:50</v>
+        <v>2026/08/11 16:49:58</v>
       </c>
       <c r="E5" t="str">
-        <v>00:19:18</v>
+        <v>00:14:00</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B6">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/08/03 17:37:48</v>
+        <v>2026/08/11 17:06:05</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/08/03 18:53:32</v>
+        <v>2026/08/11 17:12:15</v>
       </c>
       <c r="E6" t="str">
-        <v>01:15:44</v>
+        <v>00:06:10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B7">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/08/03 22:30:15</v>
+        <v>2026/08/11 21:04:07</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/08/03 22:31:24</v>
+        <v>2026/08/11 21:07:44</v>
       </c>
       <c r="E7" t="str">
-        <v>00:01:09</v>
+        <v>00:03:37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B8">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/08/04 16:06:38</v>
+        <v>2026/08/11 21:28:58</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/08/04 16:10:55</v>
+        <v>2026/08/11 21:58:42</v>
       </c>
       <c r="E8" t="str">
-        <v>00:04:17</v>
+        <v>00:29:44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B9">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/08/04 16:38:16</v>
+        <v>2026/08/11 22:36:52</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/08/04 16:49:22</v>
+        <v>2026/08/11 22:46:23</v>
       </c>
       <c r="E9" t="str">
-        <v>00:11:06</v>
+        <v>00:09:31</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B10">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/08/04 18:22:28</v>
+        <v>2026/08/11 23:19:33</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/08/04 18:27:40</v>
+        <v>2026/08/11 23:25:41</v>
       </c>
       <c r="E10" t="str">
-        <v>00:05:12</v>
+        <v>00:06:08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B11">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/08/04 20:15:29</v>
+        <v>2026/08/12 15:42:00</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/08/04 20:26:49</v>
+        <v>2026/08/12 15:44:08</v>
       </c>
       <c r="E11" t="str">
-        <v>00:11:20</v>
+        <v>00:02:08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B12">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/08/05 13:09:08</v>
+        <v>2026/08/12 16:04:25</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/08/05 13:26:56</v>
+        <v>2026/08/12 16:32:08</v>
       </c>
       <c r="E12" t="str">
-        <v>00:17:48</v>
+        <v>00:27:43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B13">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/08/05 15:09:54</v>
+        <v>2026/08/12 17:46:51</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/08/05 15:17:45</v>
+        <v>2026/08/12 18:07:43</v>
       </c>
       <c r="E13" t="str">
-        <v>00:07:51</v>
+        <v>00:20:52</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B14">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/08/05 16:43:16</v>
+        <v>2026/08/12 18:35:57</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/08/05 16:53:46</v>
+        <v>2026/08/12 18:56:49</v>
       </c>
       <c r="E14" t="str">
-        <v>00:10:30</v>
+        <v>00:20:52</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B15">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/08/05 17:15:16</v>
+        <v>2026/08/12 19:17:05</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/08/05 17:22:48</v>
+        <v>2026/08/12 19:20:20</v>
       </c>
       <c r="E15" t="str">
-        <v>00:07:32</v>
+        <v>00:03:15</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B16">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/08/06 13:20:04</v>
+        <v>2026/08/12 20:24:14</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/08/06 13:23:50</v>
+        <v>2026/08/12 20:29:09</v>
       </c>
       <c r="E16" t="str">
-        <v>00:03:46</v>
+        <v>00:04:55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B17">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/08/06 18:06:47</v>
+        <v>2026/08/12 20:41:04</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/08/06 18:08:25</v>
+        <v>2026/08/12 20:45:07</v>
       </c>
       <c r="E17" t="str">
-        <v>00:01:38</v>
+        <v>00:04:03</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B18">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/08/06 18:24:32</v>
+        <v>2026/08/12 21:33:50</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/08/06 18:48:03</v>
+        <v>2026/08/12 21:38:30</v>
       </c>
       <c r="E18" t="str">
-        <v>00:23:31</v>
+        <v>00:04:40</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B19">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/08/06 20:39:05</v>
+        <v>2026/08/12 22:01:16</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/08/06 20:45:39</v>
+        <v>2026/08/12 22:11:56</v>
       </c>
       <c r="E19" t="str">
-        <v>00:06:34</v>
+        <v>00:10:40</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B20">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/08/07 14:00:31</v>
+        <v>2026/08/12 23:12:26</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/08/07 14:16:16</v>
+        <v>2026/08/12 23:29:59</v>
       </c>
       <c r="E20" t="str">
-        <v>00:15:45</v>
+        <v>00:17:33</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B21">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/08/07 15:39:36</v>
+        <v>2026/08/13 13:16:37</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/08/07 15:49:20</v>
+        <v>2026/08/13 13:20:58</v>
       </c>
       <c r="E21" t="str">
-        <v>00:09:44</v>
+        <v>00:04:21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B22">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/08/07 16:20:55</v>
+        <v>2026/08/13 14:25:53</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/08/07 16:47:51</v>
+        <v>2026/08/13 14:31:35</v>
       </c>
       <c r="E22" t="str">
-        <v>00:26:56</v>
+        <v>00:05:42</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B23">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/08/07 17:55:13</v>
+        <v>2026/08/13 15:48:58</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/08/07 18:09:50</v>
+        <v>2026/08/13 16:19:43</v>
       </c>
       <c r="E23" t="str">
-        <v>00:14:37</v>
+        <v>00:30:45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B24">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/08/07 19:25:23</v>
+        <v>2026/08/13 16:42:54</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/08/07 19:45:36</v>
+        <v>2026/08/13 16:44:43</v>
       </c>
       <c r="E24" t="str">
-        <v>00:20:13</v>
+        <v>00:01:49</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B25">
-        <v>5209</v>
+        <v>6771</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/08/04 14:05:03</v>
+        <v>2026/08/15 23:41:07</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/08/04 14:15:15</v>
+        <v>2026/08/15 23:44:52</v>
       </c>
       <c r="E25" t="str">
-        <v>00:10:12</v>
+        <v>00:03:45</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B26">
-        <v>3860</v>
+        <v>6771</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/08/03 13:08:36</v>
+        <v>2026/08/15 23:57:10</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/08/03 13:48:22</v>
+        <v>2026/08/16 00:05:26</v>
       </c>
       <c r="E26" t="str">
-        <v>00:39:46</v>
+        <v>00:08:16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B27">
-        <v>3860</v>
+        <v>6771</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/08/03 19:48:56</v>
+        <v>2026/08/16 01:14:00</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/08/03 20:05:16</v>
+        <v>2026/08/16 01:31:12</v>
       </c>
       <c r="E27" t="str">
-        <v>00:16:20</v>
+        <v>00:17:12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B28">
-        <v>3860</v>
+        <v>6771</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/08/07 18:24:06</v>
+        <v>2026/08/16 01:42:44</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/08/07 18:25:27</v>
+        <v>2026/08/16 01:51:11</v>
       </c>
       <c r="E28" t="str">
-        <v>00:01:21</v>
+        <v>00:08:27</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B29">
-        <v>3860</v>
+        <v>6771</v>
       </c>
       <c r="C29" t="str">
-        <v>2026/08/08 14:57:00</v>
+        <v>2026/08/16 02:03:11</v>
       </c>
       <c r="D29" t="str">
-        <v>2026/08/08 15:11:59</v>
+        <v>2026/08/16 02:17:20</v>
       </c>
       <c r="E29" t="str">
-        <v>00:14:59</v>
+        <v>00:14:09</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B30">
-        <v>5651</v>
+        <v>6771</v>
       </c>
       <c r="C30" t="str">
-        <v>2026/08/04 13:51:17</v>
+        <v>2026/08/16 14:55:53</v>
       </c>
       <c r="D30" t="str">
-        <v>2026/08/04 13:57:15</v>
+        <v>2026/08/16 15:10:31</v>
       </c>
       <c r="E30" t="str">
-        <v>00:05:58</v>
+        <v>00:14:38</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B31">
-        <v>5651</v>
+        <v>6771</v>
       </c>
       <c r="C31" t="str">
-        <v>2026/08/04 19:06:00</v>
+        <v>2026/08/16 15:42:34</v>
       </c>
       <c r="D31" t="str">
-        <v>2026/08/04 19:08:08</v>
+        <v>2026/08/16 15:48:28</v>
       </c>
       <c r="E31" t="str">
-        <v>00:02:08</v>
+        <v>00:05:54</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B32">
-        <v>5651</v>
+        <v>6771</v>
       </c>
       <c r="C32" t="str">
-        <v>2026/08/07 23:24:56</v>
+        <v>2026/08/16 17:00:34</v>
       </c>
       <c r="D32" t="str">
-        <v>2026/08/07 23:37:44</v>
+        <v>2026/08/16 17:15:35</v>
       </c>
       <c r="E32" t="str">
-        <v>00:12:48</v>
+        <v>00:15:01</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B33">
-        <v>5633</v>
+        <v>5206</v>
       </c>
       <c r="C33" t="str">
-        <v>2026/08/04 16:52:54</v>
+        <v>2026/08/14 13:40:47</v>
       </c>
       <c r="D33" t="str">
-        <v>2026/08/04 17:03:20</v>
+        <v>2026/08/14 14:22:33</v>
       </c>
       <c r="E33" t="str">
-        <v>00:10:26</v>
+        <v>00:41:46</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B34">
-        <v>5633</v>
+        <v>5206</v>
       </c>
       <c r="C34" t="str">
-        <v>2026/08/05 15:30:12</v>
+        <v>2026/08/14 19:44:25</v>
       </c>
       <c r="D34" t="str">
-        <v>2026/08/05 15:31:13</v>
+        <v>2026/08/14 19:54:29</v>
       </c>
       <c r="E34" t="str">
-        <v>00:01:01</v>
+        <v>00:10:04</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B35">
-        <v>5220</v>
+        <v>3841</v>
       </c>
       <c r="C35" t="str">
-        <v>2026/08/06 14:50:16</v>
+        <v>2026/08/11 12:58:41</v>
       </c>
       <c r="D35" t="str">
-        <v>2026/08/06 15:19:34</v>
+        <v>2026/08/11 13:06:24</v>
       </c>
       <c r="E35" t="str">
-        <v>00:29:18</v>
+        <v>00:07:43</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B36">
-        <v>5245</v>
+        <v>3841</v>
       </c>
       <c r="C36" t="str">
-        <v>2026/08/07 22:20:38</v>
+        <v>2026/08/11 15:55:21</v>
       </c>
       <c r="D36" t="str">
-        <v>2026/08/07 22:21:39</v>
+        <v>2026/08/11 16:07:19</v>
       </c>
       <c r="E36" t="str">
-        <v>00:01:01</v>
+        <v>00:11:58</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B37">
-        <v>5213</v>
+        <v>3841</v>
       </c>
       <c r="C37" t="str">
-        <v>2026/08/07 14:03:01</v>
+        <v>2026/08/11 17:47:51</v>
       </c>
       <c r="D37" t="str">
-        <v>2026/08/07 14:11:34</v>
+        <v>2026/08/11 17:49:11</v>
       </c>
       <c r="E37" t="str">
-        <v>00:08:33</v>
+        <v>00:01:20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
+      </c>
+      <c r="B38">
+        <v>3841</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026/08/11 19:03:48</v>
+      </c>
+      <c r="D38" t="str">
+        <v>2026/08/11 19:14:06</v>
+      </c>
+      <c r="E38" t="str">
+        <v>00:10:18</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
+      </c>
+      <c r="B39">
+        <v>3841</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026/08/11 22:13:01</v>
+      </c>
+      <c r="D39" t="str">
+        <v>2026/08/11 23:11:57</v>
+      </c>
+      <c r="E39" t="str">
+        <v>00:58:56</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
+      </c>
+      <c r="B40">
+        <v>3841</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026/08/12 21:24:28</v>
+      </c>
+      <c r="D40" t="str">
+        <v>2026/08/12 21:32:09</v>
+      </c>
+      <c r="E40" t="str">
+        <v>00:07:41</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
+      </c>
+      <c r="B41">
+        <v>3841</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026/08/13 17:51:39</v>
+      </c>
+      <c r="D41" t="str">
+        <v>2026/08/13 17:54:45</v>
+      </c>
+      <c r="E41" t="str">
+        <v>00:03:06</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
+      </c>
+      <c r="B42">
+        <v>3841</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026/08/13 18:57:07</v>
+      </c>
+      <c r="D42" t="str">
+        <v>2026/08/13 19:01:22</v>
+      </c>
+      <c r="E42" t="str">
+        <v>00:04:15</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>MAXUS TFWK-88 (STGO)</v>
+      </c>
+      <c r="B43">
+        <v>5209</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026/08/12 15:25:35</v>
+      </c>
+      <c r="D43" t="str">
+        <v>2026/08/12 15:45:26</v>
+      </c>
+      <c r="E43" t="str">
+        <v>00:19:51</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
+      </c>
+      <c r="B44">
+        <v>3860</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026/08/10 20:38:09</v>
+      </c>
+      <c r="D44" t="str">
+        <v>2026/08/10 21:33:53</v>
+      </c>
+      <c r="E44" t="str">
+        <v>00:55:44</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
+      </c>
+      <c r="B45">
+        <v>3860</v>
+      </c>
+      <c r="C45" t="str">
+        <v>2026/08/11 17:48:12</v>
+      </c>
+      <c r="D45" t="str">
+        <v>2026/08/11 17:49:25</v>
+      </c>
+      <c r="E45" t="str">
+        <v>00:01:13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
+      </c>
+      <c r="B46">
+        <v>3860</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2026/08/13 18:40:44</v>
+      </c>
+      <c r="D46" t="str">
+        <v>2026/08/13 19:38:11</v>
+      </c>
+      <c r="E46" t="str">
+        <v>00:57:27</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
+      </c>
+      <c r="B47">
+        <v>3860</v>
+      </c>
+      <c r="C47" t="str">
+        <v>2026/08/13 21:03:29</v>
+      </c>
+      <c r="D47" t="str">
+        <v>2026/08/13 21:09:49</v>
+      </c>
+      <c r="E47" t="str">
+        <v>00:06:20</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
+      </c>
+      <c r="B48">
+        <v>3860</v>
+      </c>
+      <c r="C48" t="str">
+        <v>2026/08/14 19:29:29</v>
+      </c>
+      <c r="D48" t="str">
+        <v>2026/08/14 19:47:23</v>
+      </c>
+      <c r="E48" t="str">
+        <v>00:17:54</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>MAXUS VGVV-89 (STGO)</v>
+      </c>
+      <c r="B49">
+        <v>5633</v>
+      </c>
+      <c r="C49" t="str">
+        <v>2026/08/11 18:24:38</v>
+      </c>
+      <c r="D49" t="str">
+        <v>2026/08/11 18:28:25</v>
+      </c>
+      <c r="E49" t="str">
+        <v>00:03:47</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B50">
+        <v>5220</v>
+      </c>
+      <c r="C50" t="str">
+        <v>2026/08/10 16:19:11</v>
+      </c>
+      <c r="D50" t="str">
+        <v>2026/08/10 16:45:38</v>
+      </c>
+      <c r="E50" t="str">
+        <v>00:26:27</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B51">
+        <v>5220</v>
+      </c>
+      <c r="C51" t="str">
+        <v>2026/08/13 14:21:33</v>
+      </c>
+      <c r="D51" t="str">
+        <v>2026/08/13 15:27:01</v>
+      </c>
+      <c r="E51" t="str">
+        <v>01:05:28</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B52">
+        <v>5220</v>
+      </c>
+      <c r="C52" t="str">
+        <v>2026/08/13 15:42:53</v>
+      </c>
+      <c r="D52" t="str">
+        <v>2026/08/13 15:47:24</v>
+      </c>
+      <c r="E52" t="str">
+        <v>00:04:31</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B53">
+        <v>5220</v>
+      </c>
+      <c r="C53" t="str">
+        <v>2026/08/13 16:51:00</v>
+      </c>
+      <c r="D53" t="str">
+        <v>2026/08/13 17:54:14</v>
+      </c>
+      <c r="E53" t="str">
+        <v>01:03:14</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B54">
+        <v>5220</v>
+      </c>
+      <c r="C54" t="str">
+        <v>2026/08/14 13:44:02</v>
+      </c>
+      <c r="D54" t="str">
+        <v>2026/08/14 14:09:40</v>
+      </c>
+      <c r="E54" t="str">
+        <v>00:25:38</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B55">
+        <v>5220</v>
+      </c>
+      <c r="C55" t="str">
+        <v>2026/08/14 14:41:17</v>
+      </c>
+      <c r="D55" t="str">
+        <v>2026/08/14 15:50:03</v>
+      </c>
+      <c r="E55" t="str">
+        <v>01:08:46</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B56">
+        <v>5635</v>
+      </c>
+      <c r="C56" t="str">
+        <v>2026/08/11 15:13:15</v>
+      </c>
+      <c r="D56" t="str">
+        <v>2026/08/11 15:13:52</v>
+      </c>
+      <c r="E56" t="str">
+        <v>00:00:37</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B57">
+        <v>5635</v>
+      </c>
+      <c r="C57" t="str">
+        <v>2026/08/13 13:42:40</v>
+      </c>
+      <c r="D57" t="str">
+        <v>2026/08/13 13:45:12</v>
+      </c>
+      <c r="E57" t="str">
+        <v>00:02:32</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B58">
+        <v>5635</v>
+      </c>
+      <c r="C58" t="str">
+        <v>2026/08/13 21:17:34</v>
+      </c>
+      <c r="D58" t="str">
+        <v>2026/08/13 21:50:41</v>
+      </c>
+      <c r="E58" t="str">
+        <v>00:33:07</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B59">
+        <v>5635</v>
+      </c>
+      <c r="C59" t="str">
+        <v>2026/08/14 01:48:19</v>
+      </c>
+      <c r="D59" t="str">
+        <v>2026/08/14 01:50:39</v>
+      </c>
+      <c r="E59" t="str">
+        <v>00:02:20</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B60">
+        <v>5635</v>
+      </c>
+      <c r="C60" t="str">
+        <v>2026/08/14 12:41:10</v>
+      </c>
+      <c r="D60" t="str">
+        <v>2026/08/14 12:41:49</v>
+      </c>
+      <c r="E60" t="str">
+        <v>00:00:39</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
         <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
-      <c r="B38">
+      <c r="B61">
         <v>5223</v>
       </c>
-      <c r="C38" t="str">
-        <v>2026/08/04 12:01:53</v>
-      </c>
-      <c r="D38" t="str">
-        <v>2026/08/04 12:05:28</v>
-      </c>
-      <c r="E38" t="str">
-        <v>00:03:35</v>
+      <c r="C61" t="str">
+        <v>2026/08/10 12:32:17</v>
+      </c>
+      <c r="D61" t="str">
+        <v>2026/08/10 12:34:28</v>
+      </c>
+      <c r="E61" t="str">
+        <v>00:02:11</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B62">
+        <v>5223</v>
+      </c>
+      <c r="C62" t="str">
+        <v>2026/08/10 13:50:53</v>
+      </c>
+      <c r="D62" t="str">
+        <v>2026/08/10 13:52:36</v>
+      </c>
+      <c r="E62" t="str">
+        <v>00:01:43</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B63">
+        <v>5223</v>
+      </c>
+      <c r="C63" t="str">
+        <v>2026/08/14 18:34:00</v>
+      </c>
+      <c r="D63" t="str">
+        <v>2026/08/14 18:43:00</v>
+      </c>
+      <c r="E63" t="str">
+        <v>00:09:00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E63"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1077,13 +1502,13 @@
         <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-08-04</v>
+        <v>2026-08-10</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
-        <v>00:08:09</v>
+        <v>00:14:26</v>
       </c>
     </row>
     <row r="3">
@@ -1091,263 +1516,333 @@
         <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-11</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D3" t="str">
-        <v>00:10:41</v>
+        <v>01:16:52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-08-03</v>
+        <v>2026-08-12</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D4" t="str">
-        <v>01:50:07</v>
+        <v>01:56:41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-08-04</v>
+        <v>2026-08-13</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="str">
-        <v>00:31:55</v>
+        <v>00:42:37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-08-05</v>
+        <v>2026-08-15</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" t="str">
-        <v>00:43:41</v>
+        <v>00:12:01</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-08-06</v>
+        <v>2026-08-16</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D7" t="str">
-        <v>00:35:29</v>
+        <v>01:15:21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D8" t="str">
-        <v>01:27:15</v>
+        <v>00:51:50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-04</v>
+        <v>2026-08-11</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D9" t="str">
-        <v>00:10:12</v>
+        <v>01:30:15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-08-03</v>
+        <v>2026-08-12</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="str">
-        <v>00:56:06</v>
+        <v>00:07:41</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-13</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="str">
-        <v>00:01:21</v>
+        <v>00:07:21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-08-08</v>
+        <v>2026-08-12</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="str">
-        <v>00:14:59</v>
+        <v>00:19:51</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-08-04</v>
+        <v>2026-08-10</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="str">
-        <v>00:08:06</v>
+        <v>00:55:44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-11</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:12:48</v>
+        <v>00:01:13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-08-04</v>
+        <v>2026-08-13</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="str">
-        <v>00:10:26</v>
+        <v>01:03:47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-08-05</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="str">
-        <v>00:01:01</v>
+        <v>00:17:54</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-08-06</v>
+        <v>2026-08-11</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="str">
-        <v>00:29:18</v>
+        <v>00:03:47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-10</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="str">
-        <v>00:01:01</v>
+        <v>00:26:27</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-08-07</v>
+        <v>2026-08-13</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="str">
-        <v>00:08:33</v>
+        <v>02:13:13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20" t="str">
+        <v>01:34:24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="str">
+        <v>00:00:37</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="str">
+        <v>00:35:39</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23" t="str">
+        <v>00:02:59</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
-      <c r="B20" t="str">
-        <v>2026-08-04</v>
-      </c>
-      <c r="C20">
+      <c r="B24" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" t="str">
+        <v>00:03:54</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="C25">
         <v>1</v>
       </c>
-      <c r="D20" t="str">
-        <v>00:03:35</v>
+      <c r="D25" t="str">
+        <v>00:09:00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1365,54 +1860,54 @@
         <v>FORD RANGER VYVC-65 (ANF)</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="C2" t="str">
-        <v>00:18:50</v>
+        <v>05:37:58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>05:08:27</v>
+        <v>00:51:50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (ANTOFA)</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C4" t="str">
-        <v>00:10:12</v>
+        <v>01:45:17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>01:12:26</v>
+        <v>00:19:51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (ANTOFA)</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" t="str">
-        <v>00:20:54</v>
+        <v>02:18:38</v>
       </c>
     </row>
     <row r="7">
@@ -1420,10 +1915,10 @@
         <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>00:11:27</v>
+        <v>00:03:47</v>
       </c>
     </row>
     <row r="8">
@@ -1431,48 +1926,37 @@
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C8" t="str">
-        <v>00:29:18</v>
+        <v>04:14:04</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MITSUBISHI VDYZ-59 (Copiapo)</v>
+        <v>MITSUBISHI VDYY-82 (ANTOFA)</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C9" t="str">
-        <v>00:01:01</v>
+        <v>00:39:15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="str">
-        <v>00:08:33</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
-      <c r="C11" t="str">
-        <v>00:03:35</v>
+        <v>00:12:54</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-08-24 → 2026-08-30
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,456 +420,626 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD RANGER VYVC-51 (ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2">
         <v>6767</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/08/17 18:01:23</v>
+        <v>2026/08/25 18:46:33</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/08/17 18:07:33</v>
+        <v>2026/08/25 18:52:12</v>
       </c>
       <c r="E2" t="str">
-        <v>00:06:10</v>
+        <v>00:05:39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/08/20 23:05:10</v>
+        <v>2026/08/27 22:24:42</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/08/20 23:10:35</v>
+        <v>2026/08/27 22:39:11</v>
       </c>
       <c r="E3" t="str">
-        <v>00:05:25</v>
+        <v>00:14:29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4">
         <v>6771</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/08/21 23:18:31</v>
+        <v>2026/08/25 13:24:09</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/08/21 23:21:16</v>
+        <v>2026/08/25 13:27:40</v>
       </c>
       <c r="E4" t="str">
-        <v>00:02:45</v>
+        <v>00:03:31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5">
         <v>6771</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/08/23 19:13:28</v>
+        <v>2026/08/25 13:40:58</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/08/23 19:33:14</v>
+        <v>2026/08/25 13:43:28</v>
       </c>
       <c r="E5" t="str">
-        <v>00:19:46</v>
+        <v>00:02:30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B6">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/08/19 14:06:53</v>
+        <v>2026/08/27 17:08:55</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/08/19 14:21:22</v>
+        <v>2026/08/27 17:10:30</v>
       </c>
       <c r="E6" t="str">
-        <v>00:14:29</v>
+        <v>00:01:35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B7">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/08/19 14:32:55</v>
+        <v>2026/08/28 14:33:42</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/08/19 14:59:55</v>
+        <v>2026/08/28 14:52:33</v>
       </c>
       <c r="E7" t="str">
-        <v>00:27:00</v>
+        <v>00:18:51</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B8">
-        <v>3841</v>
+        <v>6771</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/08/19 15:28:00</v>
+        <v>2026/08/28 15:07:43</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/08/19 15:42:42</v>
+        <v>2026/08/28 15:13:59</v>
       </c>
       <c r="E8" t="str">
-        <v>00:14:42</v>
+        <v>00:06:16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B9">
         <v>3841</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/08/19 18:58:56</v>
+        <v>2026/08/24 15:36:56</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/08/19 19:06:36</v>
+        <v>2026/08/24 16:54:01</v>
       </c>
       <c r="E9" t="str">
-        <v>00:07:40</v>
+        <v>01:17:05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B10">
         <v>3841</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/08/19 21:38:08</v>
+        <v>2026/08/24 20:30:04</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/08/19 21:40:30</v>
+        <v>2026/08/24 20:33:35</v>
       </c>
       <c r="E10" t="str">
-        <v>00:02:22</v>
+        <v>00:03:31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B11">
         <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/08/20 13:05:42</v>
+        <v>2026/08/25 15:34:34</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/08/20 13:19:33</v>
+        <v>2026/08/25 15:56:16</v>
       </c>
       <c r="E11" t="str">
-        <v>00:13:51</v>
+        <v>00:21:42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B12">
         <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/08/20 16:32:44</v>
+        <v>2026/08/25 16:08:47</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/08/20 16:33:54</v>
+        <v>2026/08/25 16:45:56</v>
       </c>
       <c r="E12" t="str">
-        <v>00:01:10</v>
+        <v>00:37:09</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B13">
         <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/08/20 16:55:27</v>
+        <v>2026/08/25 19:44:08</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/08/20 17:00:40</v>
+        <v>2026/08/25 19:45:44</v>
       </c>
       <c r="E13" t="str">
-        <v>00:05:13</v>
+        <v>00:01:36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B14">
         <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/08/20 17:53:10</v>
+        <v>2026/08/25 19:58:19</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/08/20 18:02:44</v>
+        <v>2026/08/25 20:29:14</v>
       </c>
       <c r="E14" t="str">
-        <v>00:09:34</v>
+        <v>00:30:55</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B15">
         <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/08/20 18:38:25</v>
+        <v>2026/08/26 13:09:15</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/08/20 18:51:26</v>
+        <v>2026/08/26 13:35:14</v>
       </c>
       <c r="E15" t="str">
-        <v>00:13:01</v>
+        <v>00:25:59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B16">
         <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/08/20 19:03:36</v>
+        <v>2026/08/26 14:35:12</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/08/20 19:10:57</v>
+        <v>2026/08/26 14:38:53</v>
       </c>
       <c r="E16" t="str">
-        <v>00:07:21</v>
+        <v>00:03:41</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B17">
         <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/08/20 23:42:43</v>
+        <v>2026/08/26 15:04:42</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/08/20 23:45:05</v>
+        <v>2026/08/26 15:09:44</v>
       </c>
       <c r="E17" t="str">
-        <v>00:02:22</v>
+        <v>00:05:02</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B18">
         <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/08/22 13:31:30</v>
+        <v>2026/08/26 15:41:42</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/08/22 13:53:23</v>
+        <v>2026/08/26 15:59:54</v>
       </c>
       <c r="E18" t="str">
-        <v>00:21:53</v>
+        <v>00:18:12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B19">
         <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/08/22 14:15:49</v>
+        <v>2026/08/26 17:30:41</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/08/22 14:57:52</v>
+        <v>2026/08/26 17:37:25</v>
       </c>
       <c r="E19" t="str">
-        <v>00:42:03</v>
+        <v>00:06:44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B20">
         <v>3841</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/08/22 15:24:03</v>
+        <v>2026/08/26 17:47:38</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/08/22 16:29:29</v>
+        <v>2026/08/26 18:21:04</v>
       </c>
       <c r="E20" t="str">
-        <v>01:05:26</v>
+        <v>00:33:26</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B21">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/08/17 17:00:59</v>
+        <v>2026/08/26 18:33:06</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/08/17 17:04:13</v>
+        <v>2026/08/26 18:35:12</v>
       </c>
       <c r="E21" t="str">
-        <v>00:03:14</v>
+        <v>00:02:06</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B22">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/08/17 19:54:22</v>
+        <v>2026/08/26 18:45:17</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/08/17 20:39:30</v>
+        <v>2026/08/26 18:53:27</v>
       </c>
       <c r="E22" t="str">
-        <v>00:45:08</v>
+        <v>00:08:10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B23">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/08/18 14:10:56</v>
+        <v>2026/08/26 19:34:39</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/08/18 14:18:57</v>
+        <v>2026/08/26 19:57:57</v>
       </c>
       <c r="E23" t="str">
-        <v>00:08:01</v>
+        <v>00:23:18</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B24">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/08/18 15:12:34</v>
+        <v>2026/08/27 14:57:33</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/08/18 15:15:19</v>
+        <v>2026/08/27 14:59:13</v>
       </c>
       <c r="E24" t="str">
-        <v>00:02:45</v>
+        <v>00:01:40</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B25">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/08/20 17:41:03</v>
+        <v>2026/08/27 15:25:41</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/08/20 17:43:49</v>
+        <v>2026/08/27 15:32:30</v>
       </c>
       <c r="E25" t="str">
-        <v>00:02:46</v>
+        <v>00:06:49</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B26">
-        <v>3860</v>
+        <v>3841</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/08/21 13:24:18</v>
+        <v>2026/08/27 16:30:24</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/08/21 13:30:09</v>
+        <v>2026/08/27 17:11:16</v>
       </c>
       <c r="E26" t="str">
-        <v>00:05:51</v>
+        <v>00:40:52</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B27">
+        <v>3841</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2026/08/27 18:32:27</v>
+      </c>
+      <c r="D27" t="str">
+        <v>2026/08/27 18:37:30</v>
+      </c>
+      <c r="E27" t="str">
+        <v>00:05:03</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B28">
+        <v>3841</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2026/08/28 13:16:18</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2026/08/28 13:17:18</v>
+      </c>
+      <c r="E28" t="str">
+        <v>00:01:00</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B29">
+        <v>3841</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2026/08/28 14:06:18</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2026/08/28 14:15:42</v>
+      </c>
+      <c r="E29" t="str">
+        <v>00:09:24</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B30">
+        <v>3841</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2026/08/28 15:21:29</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2026/08/28 15:37:15</v>
+      </c>
+      <c r="E30" t="str">
+        <v>00:15:46</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B31">
+        <v>3841</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2026/08/28 16:45:25</v>
+      </c>
+      <c r="D31" t="str">
+        <v>2026/08/28 17:17:44</v>
+      </c>
+      <c r="E31" t="str">
+        <v>00:32:19</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B32">
+        <v>3841</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2026/08/28 19:50:24</v>
+      </c>
+      <c r="D32" t="str">
+        <v>2026/08/28 20:03:33</v>
+      </c>
+      <c r="E32" t="str">
+        <v>00:13:09</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B33">
+        <v>3841</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026/08/28 20:20:50</v>
+      </c>
+      <c r="D33" t="str">
+        <v>2026/08/28 20:49:01</v>
+      </c>
+      <c r="E33" t="str">
+        <v>00:28:11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B34">
+        <v>3860</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2026/08/26 15:09:45</v>
+      </c>
+      <c r="D34" t="str">
+        <v>2026/08/26 15:13:39</v>
+      </c>
+      <c r="E34" t="str">
+        <v>00:03:54</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B35">
+        <v>5651</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026/08/24 11:22:30</v>
+      </c>
+      <c r="D35" t="str">
+        <v>2026/08/24 11:43:52</v>
+      </c>
+      <c r="E35" t="str">
+        <v>00:21:22</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
-      <c r="B27">
+      <c r="B36">
         <v>5220</v>
       </c>
-      <c r="C27" t="str">
-        <v>2026/08/18 19:53:59</v>
-      </c>
-      <c r="D27" t="str">
-        <v>2026/08/18 20:06:55</v>
-      </c>
-      <c r="E27" t="str">
-        <v>00:12:56</v>
+      <c r="C36" t="str">
+        <v>2026/08/28 19:12:12</v>
+      </c>
+      <c r="D36" t="str">
+        <v>2026/08/28 19:14:33</v>
+      </c>
+      <c r="E36" t="str">
+        <v>00:02:21</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>PEUGEOT SRTR-81 (STGO)</v>
+      </c>
+      <c r="B37">
+        <v>5213</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026/08/24 12:28:41</v>
+      </c>
+      <c r="D37" t="str">
+        <v>2026/08/24 12:35:00</v>
+      </c>
+      <c r="E37" t="str">
+        <v>00:06:19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -887,182 +1057,210 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD RANGER VYVC-51 (ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-25</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>00:06:10</v>
+        <v>00:05:39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-27</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>00:05:25</v>
+        <v>00:14:29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-25</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="str">
-        <v>00:02:45</v>
+        <v>00:06:01</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-27</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>00:19:46</v>
+        <v>00:01:35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-08-19</v>
+        <v>2026-08-28</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6" t="str">
-        <v>01:06:13</v>
+        <v>00:25:07</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-24</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D7" t="str">
-        <v>00:52:32</v>
+        <v>01:20:36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-25</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" t="str">
-        <v>02:09:22</v>
+        <v>01:31:22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17</v>
+        <v>2026-08-26</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D9" t="str">
-        <v>00:48:22</v>
+        <v>02:06:38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-27</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" t="str">
-        <v>00:10:46</v>
+        <v>00:54:24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-28</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D11" t="str">
-        <v>00:02:46</v>
+        <v>01:39:49</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-26</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="str">
-        <v>00:05:51</v>
+        <v>00:03:54</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-24</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="str">
-        <v>00:12:56</v>
+        <v>00:21:22</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-08-28</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="str">
+        <v>00:02:21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PEUGEOT SRTR-81 (STGO)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="str">
+        <v>00:06:19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1077,62 +1275,84 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD RANGER VYVC-51 (ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>00:06:10</v>
+        <v>00:20:08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD RANGER VYVC-65 (ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="str">
-        <v>00:27:56</v>
+        <v>00:32:43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS SRYB-26 (ANTOFA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C4" t="str">
-        <v>04:08:07</v>
+        <v>07:32:49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS TYTC-88 (ANTOFA)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>01:07:45</v>
+        <v>00:03:54</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="str">
-        <v>00:12:56</v>
+        <v>00:21:22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="str">
+        <v>00:02:21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PEUGEOT SRTR-81 (STGO)</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="str">
+        <v>00:06:19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-09-14 → 2026-09-20
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,19 +420,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>6767</v>
+        <v>6766</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/08/25 18:46:33</v>
+        <v>2026/09/18 17:03:35</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/08/25 18:52:12</v>
+        <v>2026/09/18 17:09:21</v>
       </c>
       <c r="E2" t="str">
-        <v>00:05:39</v>
+        <v>00:05:46</v>
       </c>
     </row>
     <row r="3">
@@ -443,47 +443,47 @@
         <v>6767</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/08/27 22:24:42</v>
+        <v>2026/09/15 22:06:56</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/08/27 22:39:11</v>
+        <v>2026/09/15 22:09:13</v>
       </c>
       <c r="E3" t="str">
-        <v>00:14:29</v>
+        <v>00:02:17</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/08/25 13:24:09</v>
+        <v>2026/09/15 22:19:34</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/08/25 13:27:40</v>
+        <v>2026/09/15 22:26:52</v>
       </c>
       <c r="E4" t="str">
-        <v>00:03:31</v>
+        <v>00:07:18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B5">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/08/25 13:40:58</v>
+        <v>2026/09/16 10:57:34</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/08/25 13:43:28</v>
+        <v>2026/09/16 10:59:39</v>
       </c>
       <c r="E5" t="str">
-        <v>00:02:30</v>
+        <v>00:02:05</v>
       </c>
     </row>
     <row r="6">
@@ -494,47 +494,47 @@
         <v>6771</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/08/27 17:08:55</v>
+        <v>2026/09/16 11:31:05</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/08/27 17:10:30</v>
+        <v>2026/09/16 11:32:22</v>
       </c>
       <c r="E6" t="str">
-        <v>00:01:35</v>
+        <v>00:01:17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B7">
-        <v>6771</v>
+        <v>5206</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/08/28 14:33:42</v>
+        <v>2026/09/15 14:11:16</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/08/28 14:52:33</v>
+        <v>2026/09/15 14:32:41</v>
       </c>
       <c r="E7" t="str">
-        <v>00:18:51</v>
+        <v>00:21:25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8">
-        <v>6771</v>
+        <v>3841</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/08/28 15:07:43</v>
+        <v>2026/09/14 12:27:22</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/08/28 15:13:59</v>
+        <v>2026/09/14 13:09:56</v>
       </c>
       <c r="E8" t="str">
-        <v>00:06:16</v>
+        <v>00:42:34</v>
       </c>
     </row>
     <row r="9">
@@ -545,13 +545,13 @@
         <v>3841</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/08/24 15:36:56</v>
+        <v>2026/09/14 16:15:07</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/08/24 16:54:01</v>
+        <v>2026/09/14 19:49:21</v>
       </c>
       <c r="E9" t="str">
-        <v>01:17:05</v>
+        <v>03:34:14</v>
       </c>
     </row>
     <row r="10">
@@ -562,13 +562,13 @@
         <v>3841</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/08/24 20:30:04</v>
+        <v>2026/09/15 17:16:33</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/08/24 20:33:35</v>
+        <v>2026/09/15 17:40:29</v>
       </c>
       <c r="E10" t="str">
-        <v>00:03:31</v>
+        <v>00:23:56</v>
       </c>
     </row>
     <row r="11">
@@ -579,13 +579,13 @@
         <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/08/25 15:34:34</v>
+        <v>2026/09/15 18:00:52</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/08/25 15:56:16</v>
+        <v>2026/09/15 18:46:40</v>
       </c>
       <c r="E11" t="str">
-        <v>00:21:42</v>
+        <v>00:45:48</v>
       </c>
     </row>
     <row r="12">
@@ -596,13 +596,13 @@
         <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/08/25 16:08:47</v>
+        <v>2026/09/15 18:57:49</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/08/25 16:45:56</v>
+        <v>2026/09/15 19:44:06</v>
       </c>
       <c r="E12" t="str">
-        <v>00:37:09</v>
+        <v>00:46:17</v>
       </c>
     </row>
     <row r="13">
@@ -613,13 +613,13 @@
         <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/08/25 19:44:08</v>
+        <v>2026/09/16 12:14:14</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/08/25 19:45:44</v>
+        <v>2026/09/16 12:19:59</v>
       </c>
       <c r="E13" t="str">
-        <v>00:01:36</v>
+        <v>00:05:45</v>
       </c>
     </row>
     <row r="14">
@@ -630,13 +630,13 @@
         <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/08/25 19:58:19</v>
+        <v>2026/09/16 13:59:32</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/08/25 20:29:14</v>
+        <v>2026/09/16 14:45:48</v>
       </c>
       <c r="E14" t="str">
-        <v>00:30:55</v>
+        <v>00:46:16</v>
       </c>
     </row>
     <row r="15">
@@ -647,13 +647,13 @@
         <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/08/26 13:09:15</v>
+        <v>2026/09/16 14:58:12</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/08/26 13:35:14</v>
+        <v>2026/09/16 15:18:32</v>
       </c>
       <c r="E15" t="str">
-        <v>00:25:59</v>
+        <v>00:20:20</v>
       </c>
     </row>
     <row r="16">
@@ -664,13 +664,13 @@
         <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/08/26 14:35:12</v>
+        <v>2026/09/16 17:36:02</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/08/26 14:38:53</v>
+        <v>2026/09/16 18:25:11</v>
       </c>
       <c r="E16" t="str">
-        <v>00:03:41</v>
+        <v>00:49:09</v>
       </c>
     </row>
     <row r="17">
@@ -681,13 +681,13 @@
         <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/08/26 15:04:42</v>
+        <v>2026/09/16 18:47:15</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/08/26 15:09:44</v>
+        <v>2026/09/16 19:17:15</v>
       </c>
       <c r="E17" t="str">
-        <v>00:05:02</v>
+        <v>00:30:00</v>
       </c>
     </row>
     <row r="18">
@@ -698,13 +698,13 @@
         <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/08/26 15:41:42</v>
+        <v>2026/09/17 12:58:12</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/08/26 15:59:54</v>
+        <v>2026/09/17 14:01:16</v>
       </c>
       <c r="E18" t="str">
-        <v>00:18:12</v>
+        <v>01:03:04</v>
       </c>
     </row>
     <row r="19">
@@ -715,13 +715,13 @@
         <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/08/26 17:30:41</v>
+        <v>2026/09/17 14:17:22</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/08/26 17:37:25</v>
+        <v>2026/09/17 14:32:39</v>
       </c>
       <c r="E19" t="str">
-        <v>00:06:44</v>
+        <v>00:15:17</v>
       </c>
     </row>
     <row r="20">
@@ -732,314 +732,246 @@
         <v>3841</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/08/26 17:47:38</v>
+        <v>2026/09/17 15:26:20</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/08/26 18:21:04</v>
+        <v>2026/09/17 15:46:32</v>
       </c>
       <c r="E20" t="str">
-        <v>00:33:26</v>
+        <v>00:20:12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
       </c>
       <c r="B21">
-        <v>3841</v>
+        <v>4936</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/08/26 18:33:06</v>
+        <v>2026/09/14 11:36:48</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/08/26 18:35:12</v>
+        <v>2026/09/14 11:55:49</v>
       </c>
       <c r="E21" t="str">
-        <v>00:02:06</v>
+        <v>00:19:01</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B22">
-        <v>3841</v>
+        <v>5211</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/08/26 18:45:17</v>
+        <v>2026/09/15 15:22:54</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/08/26 18:53:27</v>
+        <v>2026/09/15 15:43:13</v>
       </c>
       <c r="E22" t="str">
-        <v>00:08:10</v>
+        <v>00:20:19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B23">
-        <v>3841</v>
+        <v>3860</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/08/26 19:34:39</v>
+        <v>2026/09/14 19:51:42</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/08/26 19:57:57</v>
+        <v>2026/09/14 19:59:18</v>
       </c>
       <c r="E23" t="str">
-        <v>00:23:18</v>
+        <v>00:07:36</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B24">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/08/27 14:57:33</v>
+        <v>2026/09/19 18:52:14</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/08/27 14:59:13</v>
+        <v>2026/09/19 19:02:16</v>
       </c>
       <c r="E24" t="str">
-        <v>00:01:40</v>
+        <v>00:10:02</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B25">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/08/27 15:25:41</v>
+        <v>2026/09/14 13:39:54</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/08/27 15:32:30</v>
+        <v>2026/09/14 13:42:13</v>
       </c>
       <c r="E25" t="str">
-        <v>00:06:49</v>
+        <v>00:02:19</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B26">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/08/27 16:30:24</v>
+        <v>2026/09/15 14:05:06</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/08/27 17:11:16</v>
+        <v>2026/09/15 14:52:35</v>
       </c>
       <c r="E26" t="str">
-        <v>00:40:52</v>
+        <v>00:47:29</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B27">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/08/27 18:32:27</v>
+        <v>2026/09/17 12:47:44</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/08/27 18:37:30</v>
+        <v>2026/09/17 12:49:05</v>
       </c>
       <c r="E27" t="str">
-        <v>00:05:03</v>
+        <v>00:01:21</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B28">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/08/28 13:16:18</v>
+        <v>2026/09/17 12:59:58</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/08/28 13:17:18</v>
+        <v>2026/09/17 13:07:41</v>
       </c>
       <c r="E28" t="str">
-        <v>00:01:00</v>
+        <v>00:07:43</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B29">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C29" t="str">
-        <v>2026/08/28 14:06:18</v>
+        <v>2026/09/17 13:27:44</v>
       </c>
       <c r="D29" t="str">
-        <v>2026/08/28 14:15:42</v>
+        <v>2026/09/17 13:56:44</v>
       </c>
       <c r="E29" t="str">
-        <v>00:09:24</v>
+        <v>00:29:00</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B30">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C30" t="str">
-        <v>2026/08/28 15:21:29</v>
+        <v>2026/09/17 14:06:43</v>
       </c>
       <c r="D30" t="str">
-        <v>2026/08/28 15:37:15</v>
+        <v>2026/09/17 15:03:21</v>
       </c>
       <c r="E30" t="str">
-        <v>00:15:46</v>
+        <v>00:56:38</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B31">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C31" t="str">
-        <v>2026/08/28 16:45:25</v>
+        <v>2026/09/17 15:14:20</v>
       </c>
       <c r="D31" t="str">
-        <v>2026/08/28 17:17:44</v>
+        <v>2026/09/17 15:38:52</v>
       </c>
       <c r="E31" t="str">
-        <v>00:32:19</v>
+        <v>00:24:32</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B32">
-        <v>3841</v>
+        <v>5223</v>
       </c>
       <c r="C32" t="str">
-        <v>2026/08/28 19:50:24</v>
+        <v>2026/09/15 20:26:43</v>
       </c>
       <c r="D32" t="str">
-        <v>2026/08/28 20:03:33</v>
+        <v>2026/09/15 20:47:04</v>
       </c>
       <c r="E32" t="str">
-        <v>00:13:09</v>
+        <v>00:20:21</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B33">
-        <v>3841</v>
+        <v>5223</v>
       </c>
       <c r="C33" t="str">
-        <v>2026/08/28 20:20:50</v>
+        <v>2026/09/15 22:14:35</v>
       </c>
       <c r="D33" t="str">
-        <v>2026/08/28 20:49:01</v>
+        <v>2026/09/15 22:23:16</v>
       </c>
       <c r="E33" t="str">
-        <v>00:28:11</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B34">
-        <v>3860</v>
-      </c>
-      <c r="C34" t="str">
-        <v>2026/08/26 15:09:45</v>
-      </c>
-      <c r="D34" t="str">
-        <v>2026/08/26 15:13:39</v>
-      </c>
-      <c r="E34" t="str">
-        <v>00:03:54</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B35">
-        <v>5651</v>
-      </c>
-      <c r="C35" t="str">
-        <v>2026/08/24 11:22:30</v>
-      </c>
-      <c r="D35" t="str">
-        <v>2026/08/24 11:43:52</v>
-      </c>
-      <c r="E35" t="str">
-        <v>00:21:22</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B36">
-        <v>5220</v>
-      </c>
-      <c r="C36" t="str">
-        <v>2026/08/28 19:12:12</v>
-      </c>
-      <c r="D36" t="str">
-        <v>2026/08/28 19:14:33</v>
-      </c>
-      <c r="E36" t="str">
-        <v>00:02:21</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B37">
-        <v>5213</v>
-      </c>
-      <c r="C37" t="str">
-        <v>2026/08/24 12:28:41</v>
-      </c>
-      <c r="D37" t="str">
-        <v>2026/08/24 12:35:00</v>
-      </c>
-      <c r="E37" t="str">
-        <v>00:06:19</v>
+        <v>00:08:41</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1057,16 +989,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-18</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>00:05:39</v>
+        <v>00:05:46</v>
       </c>
     </row>
     <row r="3">
@@ -1074,27 +1006,27 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-27</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="str">
-        <v>00:14:29</v>
+        <v>00:09:35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-16</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>00:06:01</v>
+        <v>00:02:05</v>
       </c>
     </row>
     <row r="5">
@@ -1102,27 +1034,27 @@
         <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-08-27</v>
+        <v>2026-09-16</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>00:01:35</v>
+        <v>00:01:17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="str">
-        <v>00:25:07</v>
+        <v>00:21:25</v>
       </c>
     </row>
     <row r="7">
@@ -1130,13 +1062,13 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-08-24</v>
+        <v>2026-09-14</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7" t="str">
-        <v>01:20:36</v>
+        <v>04:16:48</v>
       </c>
     </row>
     <row r="8">
@@ -1144,13 +1076,13 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" t="str">
-        <v>01:31:22</v>
+        <v>01:56:01</v>
       </c>
     </row>
     <row r="9">
@@ -1158,13 +1090,13 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-26</v>
+        <v>2026-09-16</v>
       </c>
       <c r="C9">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D9" t="str">
-        <v>02:06:38</v>
+        <v>02:31:30</v>
       </c>
     </row>
     <row r="10">
@@ -1172,95 +1104,137 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-08-27</v>
+        <v>2026-09-17</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="str">
-        <v>00:54:24</v>
+        <v>01:38:33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-14</v>
       </c>
       <c r="C11">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D11" t="str">
-        <v>01:39:49</v>
+        <v>00:19:01</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-08-26</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="str">
-        <v>00:03:54</v>
+        <v>00:20:19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-08-24</v>
+        <v>2026-09-14</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="str">
-        <v>00:21:22</v>
+        <v>00:07:36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-19</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:02:21</v>
+        <v>00:10:02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-08-24</v>
+        <v>2026-09-14</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="str">
-        <v>00:06:19</v>
+        <v>00:02:19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="str">
+        <v>00:47:29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17" t="str">
+        <v>01:59:14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="str">
+        <v>00:29:02</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1275,84 +1249,128 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>00:20:08</v>
+        <v>00:05:46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3" t="str">
-        <v>00:32:43</v>
+        <v>00:11:40</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>07:32:49</v>
+        <v>00:01:17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS SPRV-87 (STGO)</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>00:03:54</v>
+        <v>00:21:25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C6" t="str">
-        <v>00:21:22</v>
+        <v>10:22:52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>00:02:21</v>
+        <v>00:19:01</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="str">
-        <v>00:06:19</v>
+        <v>00:20:19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="str">
+        <v>00:07:36</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>00:10:02</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B11">
+        <v>7</v>
+      </c>
+      <c r="C11" t="str">
+        <v>02:49:02</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="str">
+        <v>00:29:02</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-09-21 → 2026-09-27
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -426,30 +426,30 @@
         <v>6766</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/09/18 17:03:35</v>
+        <v>2026/09/22 21:56:58</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/09/18 17:09:21</v>
+        <v>2026/09/22 22:01:40</v>
       </c>
       <c r="E2" t="str">
-        <v>00:05:46</v>
+        <v>00:04:42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>6767</v>
+        <v>6766</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/09/15 22:06:56</v>
+        <v>2026/09/23 15:35:48</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/09/15 22:09:13</v>
+        <v>2026/09/23 15:41:57</v>
       </c>
       <c r="E3" t="str">
-        <v>00:02:17</v>
+        <v>00:06:09</v>
       </c>
     </row>
     <row r="4">
@@ -460,13 +460,13 @@
         <v>6767</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/09/15 22:19:34</v>
+        <v>2026/09/21 16:37:34</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/09/15 22:26:52</v>
+        <v>2026/09/21 16:40:35</v>
       </c>
       <c r="E4" t="str">
-        <v>00:07:18</v>
+        <v>00:03:01</v>
       </c>
     </row>
     <row r="5">
@@ -477,47 +477,47 @@
         <v>6767</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/09/16 10:57:34</v>
+        <v>2026/09/22 00:16:48</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/09/16 10:59:39</v>
+        <v>2026/09/22 00:20:24</v>
       </c>
       <c r="E5" t="str">
-        <v>00:02:05</v>
+        <v>00:03:36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B6">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/09/16 11:31:05</v>
+        <v>2026/09/22 22:42:50</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/09/16 11:32:22</v>
+        <v>2026/09/22 22:52:30</v>
       </c>
       <c r="E6" t="str">
-        <v>00:01:17</v>
+        <v>00:09:40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SPRV-87 (STGO)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B7">
-        <v>5206</v>
+        <v>6771</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/09/15 14:11:16</v>
+        <v>2026/09/23 14:00:46</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/09/15 14:32:41</v>
+        <v>2026/09/23 14:02:27</v>
       </c>
       <c r="E7" t="str">
-        <v>00:21:25</v>
+        <v>00:01:41</v>
       </c>
     </row>
     <row r="8">
@@ -528,13 +528,13 @@
         <v>3841</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/09/14 12:27:22</v>
+        <v>2026/09/21 13:25:39</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/09/14 13:09:56</v>
+        <v>2026/09/21 13:36:56</v>
       </c>
       <c r="E8" t="str">
-        <v>00:42:34</v>
+        <v>00:11:17</v>
       </c>
     </row>
     <row r="9">
@@ -545,13 +545,13 @@
         <v>3841</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/09/14 16:15:07</v>
+        <v>2026/09/21 15:17:48</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/09/14 19:49:21</v>
+        <v>2026/09/21 15:23:38</v>
       </c>
       <c r="E9" t="str">
-        <v>03:34:14</v>
+        <v>00:05:50</v>
       </c>
     </row>
     <row r="10">
@@ -562,13 +562,13 @@
         <v>3841</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/09/15 17:16:33</v>
+        <v>2026/09/21 15:46:28</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/09/15 17:40:29</v>
+        <v>2026/09/21 16:38:01</v>
       </c>
       <c r="E10" t="str">
-        <v>00:23:56</v>
+        <v>00:51:33</v>
       </c>
     </row>
     <row r="11">
@@ -579,13 +579,13 @@
         <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/09/15 18:00:52</v>
+        <v>2026/09/21 18:01:18</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/09/15 18:46:40</v>
+        <v>2026/09/21 18:22:33</v>
       </c>
       <c r="E11" t="str">
-        <v>00:45:48</v>
+        <v>00:21:15</v>
       </c>
     </row>
     <row r="12">
@@ -596,13 +596,13 @@
         <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/09/15 18:57:49</v>
+        <v>2026/09/21 18:43:13</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/09/15 19:44:06</v>
+        <v>2026/09/21 18:55:13</v>
       </c>
       <c r="E12" t="str">
-        <v>00:46:17</v>
+        <v>00:12:00</v>
       </c>
     </row>
     <row r="13">
@@ -613,13 +613,13 @@
         <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/09/16 12:14:14</v>
+        <v>2026/09/21 19:08:28</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/09/16 12:19:59</v>
+        <v>2026/09/21 19:42:15</v>
       </c>
       <c r="E13" t="str">
-        <v>00:05:45</v>
+        <v>00:33:47</v>
       </c>
     </row>
     <row r="14">
@@ -630,13 +630,13 @@
         <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/09/16 13:59:32</v>
+        <v>2026/09/21 20:03:28</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/09/16 14:45:48</v>
+        <v>2026/09/21 20:52:29</v>
       </c>
       <c r="E14" t="str">
-        <v>00:46:16</v>
+        <v>00:49:01</v>
       </c>
     </row>
     <row r="15">
@@ -647,13 +647,13 @@
         <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/09/16 14:58:12</v>
+        <v>2026/09/23 12:20:33</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/09/16 15:18:32</v>
+        <v>2026/09/23 12:29:02</v>
       </c>
       <c r="E15" t="str">
-        <v>00:20:20</v>
+        <v>00:08:29</v>
       </c>
     </row>
     <row r="16">
@@ -664,13 +664,13 @@
         <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/09/16 17:36:02</v>
+        <v>2026/09/23 13:33:22</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/09/16 18:25:11</v>
+        <v>2026/09/23 13:50:23</v>
       </c>
       <c r="E16" t="str">
-        <v>00:49:09</v>
+        <v>00:17:01</v>
       </c>
     </row>
     <row r="17">
@@ -681,13 +681,13 @@
         <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/09/16 18:47:15</v>
+        <v>2026/09/23 14:54:37</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/09/16 19:17:15</v>
+        <v>2026/09/23 16:05:06</v>
       </c>
       <c r="E17" t="str">
-        <v>00:30:00</v>
+        <v>01:10:29</v>
       </c>
     </row>
     <row r="18">
@@ -698,13 +698,13 @@
         <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/09/17 12:58:12</v>
+        <v>2026/09/23 16:27:42</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/09/17 14:01:16</v>
+        <v>2026/09/23 16:55:51</v>
       </c>
       <c r="E18" t="str">
-        <v>01:03:04</v>
+        <v>00:28:09</v>
       </c>
     </row>
     <row r="19">
@@ -715,81 +715,81 @@
         <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/09/17 14:17:22</v>
+        <v>2026/09/23 17:18:56</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/09/17 14:32:39</v>
+        <v>2026/09/23 18:02:11</v>
       </c>
       <c r="E19" t="str">
-        <v>00:15:17</v>
+        <v>00:43:15</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B20">
-        <v>3841</v>
+        <v>3860</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/09/17 15:26:20</v>
+        <v>2026/09/23 16:55:23</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/09/17 15:46:32</v>
+        <v>2026/09/23 17:02:53</v>
       </c>
       <c r="E20" t="str">
-        <v>00:20:12</v>
+        <v>00:07:30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B21">
-        <v>4936</v>
+        <v>3860</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/09/14 11:36:48</v>
+        <v>2026/09/24 16:39:20</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/09/14 11:55:49</v>
+        <v>2026/09/24 17:26:29</v>
       </c>
       <c r="E21" t="str">
-        <v>00:19:01</v>
+        <v>00:47:09</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS TVVB-26 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B22">
-        <v>5211</v>
+        <v>5651</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/09/15 15:22:54</v>
+        <v>2026/09/22 17:52:33</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/09/15 15:43:13</v>
+        <v>2026/09/22 18:20:41</v>
       </c>
       <c r="E22" t="str">
-        <v>00:20:19</v>
+        <v>00:28:08</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B23">
-        <v>3860</v>
+        <v>5651</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/09/14 19:51:42</v>
+        <v>2026/09/24 15:21:22</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/09/14 19:59:18</v>
+        <v>2026/09/24 15:31:07</v>
       </c>
       <c r="E23" t="str">
-        <v>00:07:36</v>
+        <v>00:09:45</v>
       </c>
     </row>
     <row r="24">
@@ -800,47 +800,47 @@
         <v>5651</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/09/19 18:52:14</v>
+        <v>2026/09/24 18:30:07</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/09/19 19:02:16</v>
+        <v>2026/09/24 18:34:50</v>
       </c>
       <c r="E24" t="str">
-        <v>00:10:02</v>
+        <v>00:04:43</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B25">
-        <v>5220</v>
+        <v>5651</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/09/14 13:39:54</v>
+        <v>2026/09/25 16:11:54</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/09/14 13:42:13</v>
+        <v>2026/09/25 16:33:58</v>
       </c>
       <c r="E25" t="str">
-        <v>00:02:19</v>
+        <v>00:22:04</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B26">
-        <v>5220</v>
+        <v>5651</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/09/15 14:05:06</v>
+        <v>2026/09/25 17:38:53</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/09/15 14:52:35</v>
+        <v>2026/09/25 17:49:24</v>
       </c>
       <c r="E26" t="str">
-        <v>00:47:29</v>
+        <v>00:10:31</v>
       </c>
     </row>
     <row r="27">
@@ -851,13 +851,13 @@
         <v>5220</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/09/17 12:47:44</v>
+        <v>2026/09/21 13:18:29</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/09/17 12:49:05</v>
+        <v>2026/09/21 13:20:36</v>
       </c>
       <c r="E27" t="str">
-        <v>00:01:21</v>
+        <v>00:02:07</v>
       </c>
     </row>
     <row r="28">
@@ -868,98 +868,98 @@
         <v>5220</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/09/17 12:59:58</v>
+        <v>2026/09/22 14:29:03</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/09/17 13:07:41</v>
+        <v>2026/09/22 14:42:19</v>
       </c>
       <c r="E28" t="str">
-        <v>00:07:43</v>
+        <v>00:13:16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B29">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C29" t="str">
-        <v>2026/09/17 13:27:44</v>
+        <v>2026/09/25 14:17:14</v>
       </c>
       <c r="D29" t="str">
-        <v>2026/09/17 13:56:44</v>
+        <v>2026/09/25 14:25:33</v>
       </c>
       <c r="E29" t="str">
-        <v>00:29:00</v>
+        <v>00:08:19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B30">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C30" t="str">
-        <v>2026/09/17 14:06:43</v>
+        <v>2026/09/25 14:41:03</v>
       </c>
       <c r="D30" t="str">
-        <v>2026/09/17 15:03:21</v>
+        <v>2026/09/25 15:03:19</v>
       </c>
       <c r="E30" t="str">
-        <v>00:56:38</v>
+        <v>00:22:16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B31">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C31" t="str">
-        <v>2026/09/17 15:14:20</v>
+        <v>2026/09/25 18:27:57</v>
       </c>
       <c r="D31" t="str">
-        <v>2026/09/17 15:38:52</v>
+        <v>2026/09/25 18:34:13</v>
       </c>
       <c r="E31" t="str">
-        <v>00:24:32</v>
+        <v>00:06:16</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B32">
-        <v>5223</v>
+        <v>5213</v>
       </c>
       <c r="C32" t="str">
-        <v>2026/09/15 20:26:43</v>
+        <v>2026/09/27 12:41:37</v>
       </c>
       <c r="D32" t="str">
-        <v>2026/09/15 20:47:04</v>
+        <v>2026/09/27 13:16:01</v>
       </c>
       <c r="E32" t="str">
-        <v>00:20:21</v>
+        <v>00:34:24</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B33">
-        <v>5223</v>
+        <v>5213</v>
       </c>
       <c r="C33" t="str">
-        <v>2026/09/15 22:14:35</v>
+        <v>2026/09/27 13:31:51</v>
       </c>
       <c r="D33" t="str">
-        <v>2026/09/15 22:23:16</v>
+        <v>2026/09/27 13:45:40</v>
       </c>
       <c r="E33" t="str">
-        <v>00:08:41</v>
+        <v>00:13:49</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -992,27 +992,27 @@
         <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-22</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>00:05:46</v>
+        <v>00:04:42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>00:09:35</v>
+        <v>00:06:09</v>
       </c>
     </row>
     <row r="4">
@@ -1020,41 +1020,41 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-21</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>00:02:05</v>
+        <v>00:03:01</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-22</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="str">
-        <v>00:01:17</v>
+        <v>00:13:16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SPRV-87 (STGO)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="str">
-        <v>00:21:25</v>
+        <v>00:01:41</v>
       </c>
     </row>
     <row r="7">
@@ -1062,13 +1062,13 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-21</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D7" t="str">
-        <v>04:16:48</v>
+        <v>03:04:43</v>
       </c>
     </row>
     <row r="8">
@@ -1076,97 +1076,97 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" t="str">
-        <v>01:56:01</v>
+        <v>02:47:23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" t="str">
-        <v>02:31:30</v>
+        <v>00:07:30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-24</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" t="str">
-        <v>01:38:33</v>
+        <v>00:47:09</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-22</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="str">
-        <v>00:19:01</v>
+        <v>00:28:08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TVVB-26 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-24</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="str">
-        <v>00:20:19</v>
+        <v>00:14:28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-25</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>00:07:36</v>
+        <v>00:32:35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-21</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:10:02</v>
+        <v>00:02:07</v>
       </c>
     </row>
     <row r="15">
@@ -1174,67 +1174,53 @@
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-22</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="str">
-        <v>00:02:19</v>
+        <v>00:13:16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-25</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="str">
-        <v>00:47:29</v>
+        <v>00:36:51</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-27</v>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D17" t="str">
-        <v>01:59:14</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B18" t="str">
-        <v>2026-09-15</v>
-      </c>
-      <c r="C18">
-        <v>2</v>
-      </c>
-      <c r="D18" t="str">
-        <v>00:29:02</v>
+        <v>00:48:13</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1252,10 +1238,10 @@
         <v>FORD VYVC-47 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>00:05:46</v>
+        <v>00:10:51</v>
       </c>
     </row>
     <row r="3">
@@ -1266,7 +1252,7 @@
         <v>3</v>
       </c>
       <c r="C3" t="str">
-        <v>00:11:40</v>
+        <v>00:16:17</v>
       </c>
     </row>
     <row r="4">
@@ -1277,100 +1263,67 @@
         <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>00:01:17</v>
+        <v>00:01:41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS SPRV-87 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C5" t="str">
-        <v>00:21:25</v>
+        <v>05:52:06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C6" t="str">
-        <v>10:22:52</v>
+        <v>00:54:39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C7" t="str">
-        <v>00:19:01</v>
+        <v>01:15:11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS TVVB-26 (STGO)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="str">
-        <v>00:20:19</v>
+        <v>00:15:23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C9" t="str">
-        <v>00:07:36</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10" t="str">
-        <v>00:10:02</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B11">
-        <v>7</v>
-      </c>
-      <c r="C11" t="str">
-        <v>02:49:02</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="str">
-        <v>00:29:02</v>
+        <v>01:25:04</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-09-28 → 2026-10-04
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,104 +420,104 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-47 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>6766</v>
+        <v>6767</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/09/22 21:56:58</v>
+        <v>2026/09/29 18:29:00</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/09/22 22:01:40</v>
+        <v>2026/09/29 18:41:40</v>
       </c>
       <c r="E2" t="str">
-        <v>00:04:42</v>
+        <v>00:12:40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-47 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>6766</v>
+        <v>6767</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/09/23 15:35:48</v>
+        <v>2026/09/30 01:19:33</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/09/23 15:41:57</v>
+        <v>2026/09/30 01:22:16</v>
       </c>
       <c r="E3" t="str">
-        <v>00:06:09</v>
+        <v>00:02:43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>6767</v>
+        <v>6771</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/09/21 16:37:34</v>
+        <v>2026/09/30 17:42:25</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/09/21 16:40:35</v>
+        <v>2026/09/30 17:51:28</v>
       </c>
       <c r="E4" t="str">
-        <v>00:03:01</v>
+        <v>00:09:03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5">
-        <v>6767</v>
+        <v>6771</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/09/22 00:16:48</v>
+        <v>2026/10/02 12:40:15</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/09/22 00:20:24</v>
+        <v>2026/10/02 12:44:49</v>
       </c>
       <c r="E5" t="str">
-        <v>00:03:36</v>
+        <v>00:04:34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B6">
-        <v>6767</v>
+        <v>3841</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/09/22 22:42:50</v>
+        <v>2026/10/01 13:43:14</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/09/22 22:52:30</v>
+        <v>2026/10/01 13:43:17</v>
       </c>
       <c r="E6" t="str">
-        <v>00:09:40</v>
+        <v>00:00:03</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7">
-        <v>6771</v>
+        <v>3841</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/09/23 14:00:46</v>
+        <v>2026/10/01 15:39:01</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/09/23 14:02:27</v>
+        <v>2026/10/01 15:56:23</v>
       </c>
       <c r="E7" t="str">
-        <v>00:01:41</v>
+        <v>00:17:22</v>
       </c>
     </row>
     <row r="8">
@@ -528,450 +528,365 @@
         <v>3841</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/09/21 13:25:39</v>
+        <v>2026/10/01 17:25:37</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/09/21 13:36:56</v>
+        <v>2026/10/01 17:49:43</v>
       </c>
       <c r="E8" t="str">
-        <v>00:11:17</v>
+        <v>00:24:06</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B9">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/09/21 15:17:48</v>
+        <v>2026/09/28 17:49:54</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/09/21 15:23:38</v>
+        <v>2026/09/28 17:52:31</v>
       </c>
       <c r="E9" t="str">
-        <v>00:05:50</v>
+        <v>00:02:37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B10">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/09/21 15:46:28</v>
+        <v>2026/09/28 18:19:16</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/09/21 16:38:01</v>
+        <v>2026/09/28 18:20:43</v>
       </c>
       <c r="E10" t="str">
-        <v>00:51:33</v>
+        <v>00:01:27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B11">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/09/21 18:01:18</v>
+        <v>2026/09/29 15:37:26</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/09/21 18:22:33</v>
+        <v>2026/09/29 15:41:25</v>
       </c>
       <c r="E11" t="str">
-        <v>00:21:15</v>
+        <v>00:03:59</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B12">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/09/21 18:43:13</v>
+        <v>2026/09/30 14:11:32</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/09/21 18:55:13</v>
+        <v>2026/09/30 14:14:20</v>
       </c>
       <c r="E12" t="str">
-        <v>00:12:00</v>
+        <v>00:02:48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B13">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/09/21 19:08:28</v>
+        <v>2026/09/28 17:13:58</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/09/21 19:42:15</v>
+        <v>2026/09/28 17:14:00</v>
       </c>
       <c r="E13" t="str">
-        <v>00:33:47</v>
+        <v>00:00:02</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B14">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/09/21 20:03:28</v>
+        <v>2026/09/28 17:32:52</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/09/21 20:52:29</v>
+        <v>2026/09/28 21:21:29</v>
       </c>
       <c r="E14" t="str">
-        <v>00:49:01</v>
+        <v>03:48:37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B15">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/09/23 12:20:33</v>
+        <v>2026/09/28 21:32:01</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/09/23 12:29:02</v>
+        <v>2026/09/28 23:07:52</v>
       </c>
       <c r="E15" t="str">
-        <v>00:08:29</v>
+        <v>01:35:51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B16">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/09/23 13:33:22</v>
+        <v>2026/09/28 23:23:36</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/09/23 13:50:23</v>
+        <v>2026/09/28 23:45:54</v>
       </c>
       <c r="E16" t="str">
-        <v>00:17:01</v>
+        <v>00:22:18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B17">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/09/23 14:54:37</v>
+        <v>2026/09/29 14:23:55</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/09/23 16:05:06</v>
+        <v>2026/09/29 14:26:47</v>
       </c>
       <c r="E17" t="str">
-        <v>01:10:29</v>
+        <v>00:02:52</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B18">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/09/23 16:27:42</v>
+        <v>2026/10/01 18:28:44</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/09/23 16:55:51</v>
+        <v>2026/10/01 18:47:05</v>
       </c>
       <c r="E18" t="str">
-        <v>00:28:09</v>
+        <v>00:18:21</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B19">
-        <v>3841</v>
+        <v>5651</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/09/23 17:18:56</v>
+        <v>2026/10/01 19:19:28</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/09/23 18:02:11</v>
+        <v>2026/10/01 19:38:27</v>
       </c>
       <c r="E19" t="str">
-        <v>00:43:15</v>
+        <v>00:18:59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B20">
-        <v>3860</v>
+        <v>5651</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/09/23 16:55:23</v>
+        <v>2026/10/03 14:30:32</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/09/23 17:02:53</v>
+        <v>2026/10/03 14:34:43</v>
       </c>
       <c r="E20" t="str">
-        <v>00:07:30</v>
+        <v>00:04:11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B21">
-        <v>3860</v>
+        <v>5651</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/09/24 16:39:20</v>
+        <v>2026/10/03 16:10:44</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/09/24 17:26:29</v>
+        <v>2026/10/03 16:21:27</v>
       </c>
       <c r="E21" t="str">
-        <v>00:47:09</v>
+        <v>00:10:43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B22">
-        <v>5651</v>
+        <v>5633</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/09/22 17:52:33</v>
+        <v>2026/10/01 12:31:14</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/09/22 18:20:41</v>
+        <v>2026/10/01 12:37:47</v>
       </c>
       <c r="E22" t="str">
-        <v>00:28:08</v>
+        <v>00:06:33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B23">
-        <v>5651</v>
+        <v>5220</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/09/24 15:21:22</v>
+        <v>2026/09/29 14:09:07</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/09/24 15:31:07</v>
+        <v>2026/09/29 14:30:39</v>
       </c>
       <c r="E23" t="str">
-        <v>00:09:45</v>
+        <v>00:21:32</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B24">
-        <v>5651</v>
+        <v>5220</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/09/24 18:30:07</v>
+        <v>2026/09/29 14:41:57</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/09/24 18:34:50</v>
+        <v>2026/09/29 14:44:43</v>
       </c>
       <c r="E24" t="str">
-        <v>00:04:43</v>
+        <v>00:02:46</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B25">
-        <v>5651</v>
+        <v>5220</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/09/25 16:11:54</v>
+        <v>2026/09/29 14:54:39</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/09/25 16:33:58</v>
+        <v>2026/09/29 15:47:47</v>
       </c>
       <c r="E25" t="str">
-        <v>00:22:04</v>
+        <v>00:53:08</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B26">
-        <v>5651</v>
+        <v>5220</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/09/25 17:38:53</v>
+        <v>2026/09/29 16:03:34</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/09/25 17:49:24</v>
+        <v>2026/09/29 16:10:49</v>
       </c>
       <c r="E26" t="str">
-        <v>00:10:31</v>
+        <v>00:07:15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B27">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/09/21 13:18:29</v>
+        <v>2026/09/28 12:33:32</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/09/21 13:20:36</v>
+        <v>2026/09/28 12:36:45</v>
       </c>
       <c r="E27" t="str">
-        <v>00:02:07</v>
+        <v>00:03:13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B28">
-        <v>5220</v>
+        <v>5213</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/09/22 14:29:03</v>
+        <v>2026/09/28 13:27:56</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/09/22 14:42:19</v>
+        <v>2026/09/28 13:28:30</v>
       </c>
       <c r="E28" t="str">
-        <v>00:13:16</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B29">
-        <v>5213</v>
-      </c>
-      <c r="C29" t="str">
-        <v>2026/09/25 14:17:14</v>
-      </c>
-      <c r="D29" t="str">
-        <v>2026/09/25 14:25:33</v>
-      </c>
-      <c r="E29" t="str">
-        <v>00:08:19</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B30">
-        <v>5213</v>
-      </c>
-      <c r="C30" t="str">
-        <v>2026/09/25 14:41:03</v>
-      </c>
-      <c r="D30" t="str">
-        <v>2026/09/25 15:03:19</v>
-      </c>
-      <c r="E30" t="str">
-        <v>00:22:16</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B31">
-        <v>5213</v>
-      </c>
-      <c r="C31" t="str">
-        <v>2026/09/25 18:27:57</v>
-      </c>
-      <c r="D31" t="str">
-        <v>2026/09/25 18:34:13</v>
-      </c>
-      <c r="E31" t="str">
-        <v>00:06:16</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B32">
-        <v>5213</v>
-      </c>
-      <c r="C32" t="str">
-        <v>2026/09/27 12:41:37</v>
-      </c>
-      <c r="D32" t="str">
-        <v>2026/09/27 13:16:01</v>
-      </c>
-      <c r="E32" t="str">
-        <v>00:34:24</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B33">
-        <v>5213</v>
-      </c>
-      <c r="C33" t="str">
-        <v>2026/09/27 13:31:51</v>
-      </c>
-      <c r="D33" t="str">
-        <v>2026/09/27 13:45:40</v>
-      </c>
-      <c r="E33" t="str">
-        <v>00:13:49</v>
+        <v>00:00:34</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -989,128 +904,128 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-47 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-29</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>00:04:42</v>
+        <v>00:12:40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-47 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-23</v>
+        <v>2026-09-30</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>00:06:09</v>
+        <v>00:02:43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-30</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>00:03:01</v>
+        <v>00:09:03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-22</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>00:13:16</v>
+        <v>00:04:34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-09-23</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" t="str">
-        <v>00:01:41</v>
+        <v>00:41:31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-28</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D7" t="str">
-        <v>03:04:43</v>
+        <v>00:04:04</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-09-23</v>
+        <v>2026-09-29</v>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D8" t="str">
-        <v>02:47:23</v>
+        <v>00:03:59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-09-23</v>
+        <v>2026-09-30</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="str">
-        <v>00:07:30</v>
+        <v>00:02:48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-24</v>
+        <v>2026-09-28</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D10" t="str">
-        <v>00:47:09</v>
+        <v>05:46:48</v>
       </c>
     </row>
     <row r="11">
@@ -1118,13 +1033,13 @@
         <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-29</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="str">
-        <v>00:28:08</v>
+        <v>00:02:52</v>
       </c>
     </row>
     <row r="12">
@@ -1132,13 +1047,13 @@
         <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-09-24</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12" t="str">
-        <v>00:14:28</v>
+        <v>00:37:20</v>
       </c>
     </row>
     <row r="13">
@@ -1146,27 +1061,27 @@
         <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-09-25</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C13">
         <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>00:32:35</v>
+        <v>00:14:54</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-09-21</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:02:07</v>
+        <v>00:06:33</v>
       </c>
     </row>
     <row r="15">
@@ -1174,13 +1089,13 @@
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-29</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="str">
-        <v>00:13:16</v>
+        <v>01:24:41</v>
       </c>
     </row>
     <row r="16">
@@ -1188,32 +1103,18 @@
         <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-28</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" t="str">
-        <v>00:36:51</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
-      </c>
-      <c r="B17" t="str">
-        <v>2026-09-27</v>
-      </c>
-      <c r="C17">
-        <v>2</v>
-      </c>
-      <c r="D17" t="str">
-        <v>00:48:13</v>
+        <v>00:03:47</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1235,68 +1136,68 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-47 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>00:10:51</v>
+        <v>00:15:23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>00:16:17</v>
+        <v>00:13:37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>00:01:41</v>
+        <v>00:41:31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C5" t="str">
-        <v>05:52:06</v>
+        <v>00:10:51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C6" t="str">
-        <v>00:54:39</v>
+        <v>06:41:54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS VGVV-89 (STGO)</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>01:15:11</v>
+        <v>00:06:33</v>
       </c>
     </row>
     <row r="8">
@@ -1304,10 +1205,10 @@
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C8" t="str">
-        <v>00:15:23</v>
+        <v>01:24:41</v>
       </c>
     </row>
     <row r="9">
@@ -1315,10 +1216,10 @@
         <v>PEUGEOT SRTR-81 (STGO)</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C9" t="str">
-        <v>01:25:04</v>
+        <v>00:03:47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: reporte semana 2026-10-05 → 2026-10-11
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,13 +426,13 @@
         <v>6767</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/09/29 18:29:00</v>
+        <v>2026/10/05 13:28:44</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/09/29 18:41:40</v>
+        <v>2026/10/05 14:00:47</v>
       </c>
       <c r="E2" t="str">
-        <v>00:12:40</v>
+        <v>00:32:03</v>
       </c>
     </row>
     <row r="3">
@@ -443,450 +443,790 @@
         <v>6767</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/09/30 01:19:33</v>
+        <v>2026/10/05 14:10:48</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/09/30 01:22:16</v>
+        <v>2026/10/05 14:13:02</v>
       </c>
       <c r="E3" t="str">
-        <v>00:02:43</v>
+        <v>00:02:14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/09/30 17:42:25</v>
+        <v>2026/10/08 14:12:02</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/09/30 17:51:28</v>
+        <v>2026/10/08 14:14:21</v>
       </c>
       <c r="E4" t="str">
-        <v>00:09:03</v>
+        <v>00:02:19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B5">
-        <v>6771</v>
+        <v>6767</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/10/02 12:40:15</v>
+        <v>2026/10/08 14:40:35</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/10/02 12:44:49</v>
+        <v>2026/10/08 14:42:35</v>
       </c>
       <c r="E5" t="str">
-        <v>00:04:34</v>
+        <v>00:02:00</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B6">
-        <v>3841</v>
+        <v>6767</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/10/01 13:43:14</v>
+        <v>2026/10/08 14:52:36</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/10/01 13:43:17</v>
+        <v>2026/10/08 14:53:58</v>
       </c>
       <c r="E6" t="str">
-        <v>00:00:03</v>
+        <v>00:01:22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B7">
-        <v>3841</v>
+        <v>6767</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/10/01 15:39:01</v>
+        <v>2026/10/08 15:10:16</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/10/01 15:56:23</v>
+        <v>2026/10/08 15:13:45</v>
       </c>
       <c r="E7" t="str">
-        <v>00:17:22</v>
+        <v>00:03:29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B8">
-        <v>3841</v>
+        <v>6767</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/10/01 17:25:37</v>
+        <v>2026/10/09 17:54:21</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/10/01 17:49:43</v>
+        <v>2026/10/09 18:02:59</v>
       </c>
       <c r="E8" t="str">
-        <v>00:24:06</v>
+        <v>00:08:38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B9">
-        <v>5209</v>
+        <v>6771</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/09/28 17:49:54</v>
+        <v>2026/10/07 23:18:41</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/09/28 17:52:31</v>
+        <v>2026/10/07 23:20:55</v>
       </c>
       <c r="E9" t="str">
-        <v>00:02:37</v>
+        <v>00:02:14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>L200 VDYY-82 (CENIZA-ANF)</v>
       </c>
       <c r="B10">
-        <v>5209</v>
+        <v>5635</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/09/28 18:19:16</v>
+        <v>2026/10/05 09:42:50</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/09/28 18:20:43</v>
+        <v>2026/10/05 09:55:51</v>
       </c>
       <c r="E10" t="str">
-        <v>00:01:27</v>
+        <v>00:13:01</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B11">
-        <v>5209</v>
+        <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/09/29 15:37:26</v>
+        <v>2026/10/05 13:33:30</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/09/29 15:41:25</v>
+        <v>2026/10/05 13:41:31</v>
       </c>
       <c r="E11" t="str">
-        <v>00:03:59</v>
+        <v>00:08:01</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B12">
-        <v>5209</v>
+        <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/09/30 14:11:32</v>
+        <v>2026/10/05 16:54:14</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/09/30 14:14:20</v>
+        <v>2026/10/05 16:58:28</v>
       </c>
       <c r="E12" t="str">
-        <v>00:02:48</v>
+        <v>00:04:14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B13">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/09/28 17:13:58</v>
+        <v>2026/10/05 18:20:58</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/09/28 17:14:00</v>
+        <v>2026/10/05 18:39:26</v>
       </c>
       <c r="E13" t="str">
-        <v>00:00:02</v>
+        <v>00:18:28</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B14">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/09/28 17:32:52</v>
+        <v>2026/10/06 00:29:48</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/09/28 21:21:29</v>
+        <v>2026/10/06 00:50:56</v>
       </c>
       <c r="E14" t="str">
-        <v>03:48:37</v>
+        <v>00:21:08</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B15">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/09/28 21:32:01</v>
+        <v>2026/10/06 01:11:42</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/09/28 23:07:52</v>
+        <v>2026/10/06 01:27:08</v>
       </c>
       <c r="E15" t="str">
-        <v>01:35:51</v>
+        <v>00:15:26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B16">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/09/28 23:23:36</v>
+        <v>2026/10/06 11:46:50</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/09/28 23:45:54</v>
+        <v>2026/10/06 12:11:28</v>
       </c>
       <c r="E16" t="str">
-        <v>00:22:18</v>
+        <v>00:24:38</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B17">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/09/29 14:23:55</v>
+        <v>2026/10/06 12:53:42</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/09/29 14:26:47</v>
+        <v>2026/10/06 12:59:45</v>
       </c>
       <c r="E17" t="str">
-        <v>00:02:52</v>
+        <v>00:06:03</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B18">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/10/01 18:28:44</v>
+        <v>2026/10/06 14:03:03</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/10/01 18:47:05</v>
+        <v>2026/10/06 14:20:52</v>
       </c>
       <c r="E18" t="str">
-        <v>00:18:21</v>
+        <v>00:17:49</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B19">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/10/01 19:19:28</v>
+        <v>2026/10/06 14:37:05</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/10/01 19:38:27</v>
+        <v>2026/10/06 15:10:45</v>
       </c>
       <c r="E19" t="str">
-        <v>00:18:59</v>
+        <v>00:33:40</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B20">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/10/03 14:30:32</v>
+        <v>2026/10/06 16:06:04</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/10/03 14:34:43</v>
+        <v>2026/10/06 16:55:54</v>
       </c>
       <c r="E20" t="str">
-        <v>00:04:11</v>
+        <v>00:49:50</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B21">
-        <v>5651</v>
+        <v>3841</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/10/03 16:10:44</v>
+        <v>2026/10/07 17:49:23</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/10/03 16:21:27</v>
+        <v>2026/10/07 17:51:18</v>
       </c>
       <c r="E21" t="str">
-        <v>00:10:43</v>
+        <v>00:01:55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B22">
-        <v>5633</v>
+        <v>3841</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/10/01 12:31:14</v>
+        <v>2026/10/07 18:14:47</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/10/01 12:37:47</v>
+        <v>2026/10/07 19:08:02</v>
       </c>
       <c r="E22" t="str">
-        <v>00:06:33</v>
+        <v>00:53:15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B23">
-        <v>5220</v>
+        <v>3841</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/09/29 14:09:07</v>
+        <v>2026/10/07 19:39:43</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/09/29 14:30:39</v>
+        <v>2026/10/07 20:15:18</v>
       </c>
       <c r="E23" t="str">
-        <v>00:21:32</v>
+        <v>00:35:35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B24">
-        <v>5220</v>
+        <v>3841</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/09/29 14:41:57</v>
+        <v>2026/10/08 12:37:56</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/09/29 14:44:43</v>
+        <v>2026/10/08 13:01:01</v>
       </c>
       <c r="E24" t="str">
-        <v>00:02:46</v>
+        <v>00:23:05</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B25">
-        <v>5220</v>
+        <v>3841</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/09/29 14:54:39</v>
+        <v>2026/10/08 14:13:34</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/09/29 15:47:47</v>
+        <v>2026/10/08 14:31:46</v>
       </c>
       <c r="E25" t="str">
-        <v>00:53:08</v>
+        <v>00:18:12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B26">
-        <v>5220</v>
+        <v>3841</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/09/29 16:03:34</v>
+        <v>2026/10/08 15:43:32</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/09/29 16:10:49</v>
+        <v>2026/10/08 16:21:55</v>
       </c>
       <c r="E26" t="str">
-        <v>00:07:15</v>
+        <v>00:38:23</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B27">
-        <v>5213</v>
+        <v>3841</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/09/28 12:33:32</v>
+        <v>2026/10/08 17:04:25</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/09/28 12:36:45</v>
+        <v>2026/10/08 18:11:00</v>
       </c>
       <c r="E27" t="str">
-        <v>00:03:13</v>
+        <v>01:06:35</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B28">
-        <v>5213</v>
+        <v>3841</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/09/28 13:27:56</v>
+        <v>2026/10/08 19:29:34</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/09/28 13:28:30</v>
+        <v>2026/10/08 19:32:07</v>
       </c>
       <c r="E28" t="str">
-        <v>00:00:34</v>
+        <v>00:02:33</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B29">
+        <v>3841</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2026/10/09 14:27:50</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2026/10/09 14:28:36</v>
+      </c>
+      <c r="E29" t="str">
+        <v>00:00:46</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B30">
+        <v>3841</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2026/10/09 15:52:21</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2026/10/09 16:07:17</v>
+      </c>
+      <c r="E30" t="str">
+        <v>00:14:56</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B31">
+        <v>3841</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2026/10/09 18:34:42</v>
+      </c>
+      <c r="D31" t="str">
+        <v>2026/10/09 18:47:44</v>
+      </c>
+      <c r="E31" t="str">
+        <v>00:13:02</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B32">
+        <v>3841</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2026/10/09 19:30:27</v>
+      </c>
+      <c r="D32" t="str">
+        <v>2026/10/09 19:33:28</v>
+      </c>
+      <c r="E32" t="str">
+        <v>00:03:01</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+      </c>
+      <c r="B33">
+        <v>3841</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026/10/09 19:49:10</v>
+      </c>
+      <c r="D33" t="str">
+        <v>2026/10/09 20:14:31</v>
+      </c>
+      <c r="E33" t="str">
+        <v>00:25:21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
+      </c>
+      <c r="B34">
+        <v>4936</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2026/10/09 14:53:19</v>
+      </c>
+      <c r="D34" t="str">
+        <v>2026/10/09 14:54:58</v>
+      </c>
+      <c r="E34" t="str">
+        <v>00:01:39</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B35">
+        <v>3860</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026/10/05 22:52:35</v>
+      </c>
+      <c r="D35" t="str">
+        <v>2026/10/05 22:55:29</v>
+      </c>
+      <c r="E35" t="str">
+        <v>00:02:54</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B36">
+        <v>3860</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2026/10/06 16:51:24</v>
+      </c>
+      <c r="D36" t="str">
+        <v>2026/10/06 17:06:54</v>
+      </c>
+      <c r="E36" t="str">
+        <v>00:15:30</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B37">
+        <v>3860</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026/10/06 19:31:09</v>
+      </c>
+      <c r="D37" t="str">
+        <v>2026/10/06 19:32:18</v>
+      </c>
+      <c r="E37" t="str">
+        <v>00:01:09</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B38">
+        <v>3860</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026/10/08 11:57:37</v>
+      </c>
+      <c r="D38" t="str">
+        <v>2026/10/08 12:00:28</v>
+      </c>
+      <c r="E38" t="str">
+        <v>00:02:51</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B39">
+        <v>3860</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026/10/08 12:34:03</v>
+      </c>
+      <c r="D39" t="str">
+        <v>2026/10/08 12:57:45</v>
+      </c>
+      <c r="E39" t="str">
+        <v>00:23:42</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B40">
+        <v>3860</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026/10/08 14:32:07</v>
+      </c>
+      <c r="D40" t="str">
+        <v>2026/10/08 14:46:34</v>
+      </c>
+      <c r="E40" t="str">
+        <v>00:14:27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+      </c>
+      <c r="B41">
+        <v>3860</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026/10/08 19:08:34</v>
+      </c>
+      <c r="D41" t="str">
+        <v>2026/10/08 19:45:06</v>
+      </c>
+      <c r="E41" t="str">
+        <v>00:36:32</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B42">
+        <v>5651</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026/10/05 15:05:31</v>
+      </c>
+      <c r="D42" t="str">
+        <v>2026/10/05 15:05:50</v>
+      </c>
+      <c r="E42" t="str">
+        <v>00:00:19</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B43">
+        <v>5651</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026/10/05 15:40:19</v>
+      </c>
+      <c r="D43" t="str">
+        <v>2026/10/05 15:50:38</v>
+      </c>
+      <c r="E43" t="str">
+        <v>00:10:19</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B44">
+        <v>5651</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026/10/05 17:57:57</v>
+      </c>
+      <c r="D44" t="str">
+        <v>2026/10/05 18:00:43</v>
+      </c>
+      <c r="E44" t="str">
+        <v>00:02:46</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>MAXUS VGVV-79 (STGO MA)</v>
+      </c>
+      <c r="B45">
+        <v>5651</v>
+      </c>
+      <c r="C45" t="str">
+        <v>2026/10/05 18:24:02</v>
+      </c>
+      <c r="D45" t="str">
+        <v>2026/10/05 18:31:27</v>
+      </c>
+      <c r="E45" t="str">
+        <v>00:07:25</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B46">
+        <v>5220</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2026/10/07 17:01:50</v>
+      </c>
+      <c r="D46" t="str">
+        <v>2026/10/07 17:05:56</v>
+      </c>
+      <c r="E46" t="str">
+        <v>00:04:06</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B47">
+        <v>5220</v>
+      </c>
+      <c r="C47" t="str">
+        <v>2026/10/09 17:57:20</v>
+      </c>
+      <c r="D47" t="str">
+        <v>2026/10/09 18:26:48</v>
+      </c>
+      <c r="E47" t="str">
+        <v>00:29:28</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B48">
+        <v>5223</v>
+      </c>
+      <c r="C48" t="str">
+        <v>2026/10/07 16:06:17</v>
+      </c>
+      <c r="D48" t="str">
+        <v>2026/10/07 16:15:22</v>
+      </c>
+      <c r="E48" t="str">
+        <v>00:09:05</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -907,13 +1247,13 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
-        <v>00:12:40</v>
+        <v>00:34:17</v>
       </c>
     </row>
     <row r="3">
@@ -921,27 +1261,27 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-30</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3" t="str">
-        <v>00:02:43</v>
+        <v>00:09:10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-09-30</v>
+        <v>2026-10-09</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>00:09:03</v>
+        <v>00:08:38</v>
       </c>
     </row>
     <row r="5">
@@ -949,179 +1289,221 @@
         <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-07</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>00:04:34</v>
+        <v>00:02:14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>L200 VDYY-82 (CENIZA-ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" t="str">
-        <v>00:41:31</v>
+        <v>00:13:01</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="str">
-        <v>00:04:04</v>
+        <v>00:30:43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-06</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D8" t="str">
-        <v>00:03:59</v>
+        <v>02:48:34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-09-30</v>
+        <v>2026-10-07</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D9" t="str">
-        <v>00:02:48</v>
+        <v>01:30:45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" t="str">
-        <v>05:46:48</v>
+        <v>02:28:48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-09</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D11" t="str">
-        <v>00:02:52</v>
+        <v>00:57:06</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-09</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="str">
-        <v>00:37:20</v>
+        <v>00:01:39</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="str">
-        <v>00:14:54</v>
+        <v>00:02:54</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-06</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="str">
-        <v>00:06:33</v>
+        <v>00:16:39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C15">
         <v>4</v>
       </c>
       <c r="D15" t="str">
-        <v>01:24:41</v>
+        <v>01:17:32</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" t="str">
-        <v>00:03:47</v>
+        <v>00:20:49</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-10-07</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="str">
+        <v>00:04:06</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-10-09</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>00:29:28</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-10-07</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>00:09:05</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1139,10 +1521,10 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C2" t="str">
-        <v>00:15:23</v>
+        <v>00:52:05</v>
       </c>
     </row>
     <row r="3">
@@ -1150,81 +1532,92 @@
         <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>00:13:37</v>
+        <v>00:02:14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>L200 VDYY-82 (CENIZA-ANF)</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>00:41:31</v>
+        <v>00:13:01</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MAXUS TFWK-88 (STGO)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C5" t="str">
-        <v>00:10:51</v>
+        <v>08:15:56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TVVB-25 (CHILLAN)</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C6" t="str">
-        <v>06:41:54</v>
+        <v>00:01:39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS VGVV-89 (STGO)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C7" t="str">
-        <v>00:06:33</v>
+        <v>01:37:05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
+        <v>MAXUS VGVV-79 (STGO MA)</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
       <c r="C8" t="str">
-        <v>01:24:41</v>
+        <v>00:20:49</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PEUGEOT SRTR-81 (STGO)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" t="str">
-        <v>00:03:47</v>
+        <v>00:33:34</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PEUGEOT SVCH-53 (STGO)</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>00:09:05</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
auto: reporte semana 2026-10-12 → 2026-10-18
</commit_message>
<xml_diff>
--- a/RALENTI EXCESIVO.xlsx
+++ b/RALENTI EXCESIVO.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,19 +420,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD RANGER VYVC-38 (STGO PR)</v>
       </c>
       <c r="B2">
-        <v>6767</v>
+        <v>6769</v>
       </c>
       <c r="C2" t="str">
-        <v>2026/10/05 13:28:44</v>
+        <v>2026/10/15 18:54:20</v>
       </c>
       <c r="D2" t="str">
-        <v>2026/10/05 14:00:47</v>
+        <v>2026/10/15 20:11:02</v>
       </c>
       <c r="E2" t="str">
-        <v>00:32:03</v>
+        <v>01:16:42</v>
       </c>
     </row>
     <row r="3">
@@ -443,132 +443,132 @@
         <v>6767</v>
       </c>
       <c r="C3" t="str">
-        <v>2026/10/05 14:10:48</v>
+        <v>2026/10/15 15:28:58</v>
       </c>
       <c r="D3" t="str">
-        <v>2026/10/05 14:13:02</v>
+        <v>2026/10/15 15:35:07</v>
       </c>
       <c r="E3" t="str">
-        <v>00:02:14</v>
+        <v>00:06:09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>6767</v>
+        <v>6771</v>
       </c>
       <c r="C4" t="str">
-        <v>2026/10/08 14:12:02</v>
+        <v>2026/10/14 13:09:21</v>
       </c>
       <c r="D4" t="str">
-        <v>2026/10/08 14:14:21</v>
+        <v>2026/10/14 13:11:58</v>
       </c>
       <c r="E4" t="str">
-        <v>00:02:19</v>
+        <v>00:02:37</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5">
-        <v>6767</v>
+        <v>6771</v>
       </c>
       <c r="C5" t="str">
-        <v>2026/10/08 14:40:35</v>
+        <v>2026/10/17 22:47:38</v>
       </c>
       <c r="D5" t="str">
-        <v>2026/10/08 14:42:35</v>
+        <v>2026/10/17 22:49:55</v>
       </c>
       <c r="E5" t="str">
-        <v>00:02:00</v>
+        <v>00:02:17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B6">
-        <v>6767</v>
+        <v>3841</v>
       </c>
       <c r="C6" t="str">
-        <v>2026/10/08 14:52:36</v>
+        <v>2026/10/13 12:16:06</v>
       </c>
       <c r="D6" t="str">
-        <v>2026/10/08 14:53:58</v>
+        <v>2026/10/13 12:18:02</v>
       </c>
       <c r="E6" t="str">
-        <v>00:01:22</v>
+        <v>00:01:56</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7">
-        <v>6767</v>
+        <v>3841</v>
       </c>
       <c r="C7" t="str">
-        <v>2026/10/08 15:10:16</v>
+        <v>2026/10/13 15:46:41</v>
       </c>
       <c r="D7" t="str">
-        <v>2026/10/08 15:13:45</v>
+        <v>2026/10/13 15:54:48</v>
       </c>
       <c r="E7" t="str">
-        <v>00:03:29</v>
+        <v>00:08:07</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8">
-        <v>6767</v>
+        <v>3841</v>
       </c>
       <c r="C8" t="str">
-        <v>2026/10/09 17:54:21</v>
+        <v>2026/10/13 18:42:50</v>
       </c>
       <c r="D8" t="str">
-        <v>2026/10/09 18:02:59</v>
+        <v>2026/10/13 18:58:51</v>
       </c>
       <c r="E8" t="str">
-        <v>00:08:38</v>
+        <v>00:16:01</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B9">
-        <v>6771</v>
+        <v>3841</v>
       </c>
       <c r="C9" t="str">
-        <v>2026/10/07 23:18:41</v>
+        <v>2026/10/13 19:22:28</v>
       </c>
       <c r="D9" t="str">
-        <v>2026/10/07 23:20:55</v>
+        <v>2026/10/13 19:35:32</v>
       </c>
       <c r="E9" t="str">
-        <v>00:02:14</v>
+        <v>00:13:04</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>L200 VDYY-82 (CENIZA-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B10">
-        <v>5635</v>
+        <v>3841</v>
       </c>
       <c r="C10" t="str">
-        <v>2026/10/05 09:42:50</v>
+        <v>2026/10/13 19:58:40</v>
       </c>
       <c r="D10" t="str">
-        <v>2026/10/05 09:55:51</v>
+        <v>2026/10/13 20:03:34</v>
       </c>
       <c r="E10" t="str">
-        <v>00:13:01</v>
+        <v>00:04:54</v>
       </c>
     </row>
     <row r="11">
@@ -579,13 +579,13 @@
         <v>3841</v>
       </c>
       <c r="C11" t="str">
-        <v>2026/10/05 13:33:30</v>
+        <v>2026/10/14 12:51:00</v>
       </c>
       <c r="D11" t="str">
-        <v>2026/10/05 13:41:31</v>
+        <v>2026/10/14 12:53:00</v>
       </c>
       <c r="E11" t="str">
-        <v>00:08:01</v>
+        <v>00:02:00</v>
       </c>
     </row>
     <row r="12">
@@ -596,13 +596,13 @@
         <v>3841</v>
       </c>
       <c r="C12" t="str">
-        <v>2026/10/05 16:54:14</v>
+        <v>2026/10/14 13:06:18</v>
       </c>
       <c r="D12" t="str">
-        <v>2026/10/05 16:58:28</v>
+        <v>2026/10/14 13:24:04</v>
       </c>
       <c r="E12" t="str">
-        <v>00:04:14</v>
+        <v>00:17:46</v>
       </c>
     </row>
     <row r="13">
@@ -613,13 +613,13 @@
         <v>3841</v>
       </c>
       <c r="C13" t="str">
-        <v>2026/10/05 18:20:58</v>
+        <v>2026/10/14 14:38:11</v>
       </c>
       <c r="D13" t="str">
-        <v>2026/10/05 18:39:26</v>
+        <v>2026/10/14 15:54:37</v>
       </c>
       <c r="E13" t="str">
-        <v>00:18:28</v>
+        <v>01:16:26</v>
       </c>
     </row>
     <row r="14">
@@ -630,13 +630,13 @@
         <v>3841</v>
       </c>
       <c r="C14" t="str">
-        <v>2026/10/06 00:29:48</v>
+        <v>2026/10/14 17:32:10</v>
       </c>
       <c r="D14" t="str">
-        <v>2026/10/06 00:50:56</v>
+        <v>2026/10/14 17:39:24</v>
       </c>
       <c r="E14" t="str">
-        <v>00:21:08</v>
+        <v>00:07:14</v>
       </c>
     </row>
     <row r="15">
@@ -647,13 +647,13 @@
         <v>3841</v>
       </c>
       <c r="C15" t="str">
-        <v>2026/10/06 01:11:42</v>
+        <v>2026/10/14 18:23:38</v>
       </c>
       <c r="D15" t="str">
-        <v>2026/10/06 01:27:08</v>
+        <v>2026/10/14 18:34:56</v>
       </c>
       <c r="E15" t="str">
-        <v>00:15:26</v>
+        <v>00:11:18</v>
       </c>
     </row>
     <row r="16">
@@ -664,13 +664,13 @@
         <v>3841</v>
       </c>
       <c r="C16" t="str">
-        <v>2026/10/06 11:46:50</v>
+        <v>2026/10/14 19:24:45</v>
       </c>
       <c r="D16" t="str">
-        <v>2026/10/06 12:11:28</v>
+        <v>2026/10/14 19:36:58</v>
       </c>
       <c r="E16" t="str">
-        <v>00:24:38</v>
+        <v>00:12:13</v>
       </c>
     </row>
     <row r="17">
@@ -681,13 +681,13 @@
         <v>3841</v>
       </c>
       <c r="C17" t="str">
-        <v>2026/10/06 12:53:42</v>
+        <v>2026/10/15 13:43:29</v>
       </c>
       <c r="D17" t="str">
-        <v>2026/10/06 12:59:45</v>
+        <v>2026/10/15 13:50:47</v>
       </c>
       <c r="E17" t="str">
-        <v>00:06:03</v>
+        <v>00:07:18</v>
       </c>
     </row>
     <row r="18">
@@ -698,13 +698,13 @@
         <v>3841</v>
       </c>
       <c r="C18" t="str">
-        <v>2026/10/06 14:03:03</v>
+        <v>2026/10/15 14:37:01</v>
       </c>
       <c r="D18" t="str">
-        <v>2026/10/06 14:20:52</v>
+        <v>2026/10/15 16:01:28</v>
       </c>
       <c r="E18" t="str">
-        <v>00:17:49</v>
+        <v>01:24:27</v>
       </c>
     </row>
     <row r="19">
@@ -715,13 +715,13 @@
         <v>3841</v>
       </c>
       <c r="C19" t="str">
-        <v>2026/10/06 14:37:05</v>
+        <v>2026/10/15 16:59:04</v>
       </c>
       <c r="D19" t="str">
-        <v>2026/10/06 15:10:45</v>
+        <v>2026/10/15 17:19:00</v>
       </c>
       <c r="E19" t="str">
-        <v>00:33:40</v>
+        <v>00:19:56</v>
       </c>
     </row>
     <row r="20">
@@ -732,13 +732,13 @@
         <v>3841</v>
       </c>
       <c r="C20" t="str">
-        <v>2026/10/06 16:06:04</v>
+        <v>2026/10/15 18:40:00</v>
       </c>
       <c r="D20" t="str">
-        <v>2026/10/06 16:55:54</v>
+        <v>2026/10/15 18:44:03</v>
       </c>
       <c r="E20" t="str">
-        <v>00:49:50</v>
+        <v>00:04:03</v>
       </c>
     </row>
     <row r="21">
@@ -749,484 +749,229 @@
         <v>3841</v>
       </c>
       <c r="C21" t="str">
-        <v>2026/10/07 17:49:23</v>
+        <v>2026/10/15 19:02:02</v>
       </c>
       <c r="D21" t="str">
-        <v>2026/10/07 17:51:18</v>
+        <v>2026/10/15 19:26:40</v>
       </c>
       <c r="E21" t="str">
-        <v>00:01:55</v>
+        <v>00:24:38</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B22">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C22" t="str">
-        <v>2026/10/07 18:14:47</v>
+        <v>2026/10/16 14:02:50</v>
       </c>
       <c r="D22" t="str">
-        <v>2026/10/07 19:08:02</v>
+        <v>2026/10/16 14:10:04</v>
       </c>
       <c r="E22" t="str">
-        <v>00:53:15</v>
+        <v>00:07:14</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B23">
-        <v>3841</v>
+        <v>5209</v>
       </c>
       <c r="C23" t="str">
-        <v>2026/10/07 19:39:43</v>
+        <v>2026/10/16 15:17:00</v>
       </c>
       <c r="D23" t="str">
-        <v>2026/10/07 20:15:18</v>
+        <v>2026/10/16 15:22:24</v>
       </c>
       <c r="E23" t="str">
-        <v>00:35:35</v>
+        <v>00:05:24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B24">
-        <v>3841</v>
+        <v>5211</v>
       </c>
       <c r="C24" t="str">
-        <v>2026/10/08 12:37:56</v>
+        <v>2026/10/16 21:54:18</v>
       </c>
       <c r="D24" t="str">
-        <v>2026/10/08 13:01:01</v>
+        <v>2026/10/16 21:59:02</v>
       </c>
       <c r="E24" t="str">
-        <v>00:23:05</v>
+        <v>00:04:44</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B25">
-        <v>3841</v>
+        <v>3860</v>
       </c>
       <c r="C25" t="str">
-        <v>2026/10/08 14:13:34</v>
+        <v>2026/10/13 13:03:06</v>
       </c>
       <c r="D25" t="str">
-        <v>2026/10/08 14:31:46</v>
+        <v>2026/10/13 13:28:23</v>
       </c>
       <c r="E25" t="str">
-        <v>00:18:12</v>
+        <v>00:25:17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B26">
-        <v>3841</v>
+        <v>3860</v>
       </c>
       <c r="C26" t="str">
-        <v>2026/10/08 15:43:32</v>
+        <v>2026/10/13 14:52:25</v>
       </c>
       <c r="D26" t="str">
-        <v>2026/10/08 16:21:55</v>
+        <v>2026/10/13 15:54:36</v>
       </c>
       <c r="E26" t="str">
-        <v>00:38:23</v>
+        <v>01:02:11</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B27">
-        <v>3841</v>
+        <v>3860</v>
       </c>
       <c r="C27" t="str">
-        <v>2026/10/08 17:04:25</v>
+        <v>2026/10/13 17:31:34</v>
       </c>
       <c r="D27" t="str">
-        <v>2026/10/08 18:11:00</v>
+        <v>2026/10/13 17:54:29</v>
       </c>
       <c r="E27" t="str">
-        <v>01:06:35</v>
+        <v>00:22:55</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B28">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C28" t="str">
-        <v>2026/10/08 19:29:34</v>
+        <v>2026/10/14 14:21:37</v>
       </c>
       <c r="D28" t="str">
-        <v>2026/10/08 19:32:07</v>
+        <v>2026/10/14 14:37:02</v>
       </c>
       <c r="E28" t="str">
-        <v>00:02:33</v>
+        <v>00:15:25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B29">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C29" t="str">
-        <v>2026/10/09 14:27:50</v>
+        <v>2026/10/14 14:56:35</v>
       </c>
       <c r="D29" t="str">
-        <v>2026/10/09 14:28:36</v>
+        <v>2026/10/14 15:03:09</v>
       </c>
       <c r="E29" t="str">
-        <v>00:00:46</v>
+        <v>00:06:34</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B30">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C30" t="str">
-        <v>2026/10/09 15:52:21</v>
+        <v>2026/10/14 15:14:55</v>
       </c>
       <c r="D30" t="str">
-        <v>2026/10/09 16:07:17</v>
+        <v>2026/10/14 15:42:30</v>
       </c>
       <c r="E30" t="str">
-        <v>00:14:56</v>
+        <v>00:27:35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B31">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C31" t="str">
-        <v>2026/10/09 18:34:42</v>
+        <v>2026/10/16 15:12:48</v>
       </c>
       <c r="D31" t="str">
-        <v>2026/10/09 18:47:44</v>
+        <v>2026/10/16 16:40:38</v>
       </c>
       <c r="E31" t="str">
-        <v>00:13:02</v>
+        <v>01:27:50</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B32">
-        <v>3841</v>
+        <v>5220</v>
       </c>
       <c r="C32" t="str">
-        <v>2026/10/09 19:30:27</v>
+        <v>2026/10/16 16:50:40</v>
       </c>
       <c r="D32" t="str">
-        <v>2026/10/09 19:33:28</v>
+        <v>2026/10/16 16:52:00</v>
       </c>
       <c r="E32" t="str">
-        <v>00:03:01</v>
+        <v>00:01:20</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B33">
-        <v>3841</v>
+        <v>5223</v>
       </c>
       <c r="C33" t="str">
-        <v>2026/10/09 19:49:10</v>
+        <v>2026/10/14 13:39:51</v>
       </c>
       <c r="D33" t="str">
-        <v>2026/10/09 20:14:31</v>
+        <v>2026/10/14 13:47:48</v>
       </c>
       <c r="E33" t="str">
-        <v>00:25:21</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
-      </c>
-      <c r="B34">
-        <v>4936</v>
-      </c>
-      <c r="C34" t="str">
-        <v>2026/10/09 14:53:19</v>
-      </c>
-      <c r="D34" t="str">
-        <v>2026/10/09 14:54:58</v>
-      </c>
-      <c r="E34" t="str">
-        <v>00:01:39</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B35">
-        <v>3860</v>
-      </c>
-      <c r="C35" t="str">
-        <v>2026/10/05 22:52:35</v>
-      </c>
-      <c r="D35" t="str">
-        <v>2026/10/05 22:55:29</v>
-      </c>
-      <c r="E35" t="str">
-        <v>00:02:54</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B36">
-        <v>3860</v>
-      </c>
-      <c r="C36" t="str">
-        <v>2026/10/06 16:51:24</v>
-      </c>
-      <c r="D36" t="str">
-        <v>2026/10/06 17:06:54</v>
-      </c>
-      <c r="E36" t="str">
-        <v>00:15:30</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B37">
-        <v>3860</v>
-      </c>
-      <c r="C37" t="str">
-        <v>2026/10/06 19:31:09</v>
-      </c>
-      <c r="D37" t="str">
-        <v>2026/10/06 19:32:18</v>
-      </c>
-      <c r="E37" t="str">
-        <v>00:01:09</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B38">
-        <v>3860</v>
-      </c>
-      <c r="C38" t="str">
-        <v>2026/10/08 11:57:37</v>
-      </c>
-      <c r="D38" t="str">
-        <v>2026/10/08 12:00:28</v>
-      </c>
-      <c r="E38" t="str">
-        <v>00:02:51</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B39">
-        <v>3860</v>
-      </c>
-      <c r="C39" t="str">
-        <v>2026/10/08 12:34:03</v>
-      </c>
-      <c r="D39" t="str">
-        <v>2026/10/08 12:57:45</v>
-      </c>
-      <c r="E39" t="str">
-        <v>00:23:42</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B40">
-        <v>3860</v>
-      </c>
-      <c r="C40" t="str">
-        <v>2026/10/08 14:32:07</v>
-      </c>
-      <c r="D40" t="str">
-        <v>2026/10/08 14:46:34</v>
-      </c>
-      <c r="E40" t="str">
-        <v>00:14:27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B41">
-        <v>3860</v>
-      </c>
-      <c r="C41" t="str">
-        <v>2026/10/08 19:08:34</v>
-      </c>
-      <c r="D41" t="str">
-        <v>2026/10/08 19:45:06</v>
-      </c>
-      <c r="E41" t="str">
-        <v>00:36:32</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B42">
-        <v>5651</v>
-      </c>
-      <c r="C42" t="str">
-        <v>2026/10/05 15:05:31</v>
-      </c>
-      <c r="D42" t="str">
-        <v>2026/10/05 15:05:50</v>
-      </c>
-      <c r="E42" t="str">
-        <v>00:00:19</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B43">
-        <v>5651</v>
-      </c>
-      <c r="C43" t="str">
-        <v>2026/10/05 15:40:19</v>
-      </c>
-      <c r="D43" t="str">
-        <v>2026/10/05 15:50:38</v>
-      </c>
-      <c r="E43" t="str">
-        <v>00:10:19</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B44">
-        <v>5651</v>
-      </c>
-      <c r="C44" t="str">
-        <v>2026/10/05 17:57:57</v>
-      </c>
-      <c r="D44" t="str">
-        <v>2026/10/05 18:00:43</v>
-      </c>
-      <c r="E44" t="str">
-        <v>00:02:46</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B45">
-        <v>5651</v>
-      </c>
-      <c r="C45" t="str">
-        <v>2026/10/05 18:24:02</v>
-      </c>
-      <c r="D45" t="str">
-        <v>2026/10/05 18:31:27</v>
-      </c>
-      <c r="E45" t="str">
-        <v>00:07:25</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B46">
-        <v>5220</v>
-      </c>
-      <c r="C46" t="str">
-        <v>2026/10/07 17:01:50</v>
-      </c>
-      <c r="D46" t="str">
-        <v>2026/10/07 17:05:56</v>
-      </c>
-      <c r="E46" t="str">
-        <v>00:04:06</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B47">
-        <v>5220</v>
-      </c>
-      <c r="C47" t="str">
-        <v>2026/10/09 17:57:20</v>
-      </c>
-      <c r="D47" t="str">
-        <v>2026/10/09 18:26:48</v>
-      </c>
-      <c r="E47" t="str">
-        <v>00:29:28</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B48">
-        <v>5223</v>
-      </c>
-      <c r="C48" t="str">
-        <v>2026/10/07 16:06:17</v>
-      </c>
-      <c r="D48" t="str">
-        <v>2026/10/07 16:15:22</v>
-      </c>
-      <c r="E48" t="str">
-        <v>00:09:05</v>
+        <v>00:07:57</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1244,16 +989,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD RANGER VYVC-38 (STGO PR)</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>00:34:17</v>
+        <v>01:16:42</v>
       </c>
     </row>
     <row r="3">
@@ -1261,27 +1006,27 @@
         <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>00:09:10</v>
+        <v>00:06:09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>00:08:38</v>
+        <v>00:02:37</v>
       </c>
     </row>
     <row r="5">
@@ -1289,27 +1034,27 @@
         <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-17</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>00:02:14</v>
+        <v>00:02:17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>L200 VDYY-82 (CENIZA-ANF)</v>
+        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-13</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6" t="str">
-        <v>00:13:01</v>
+        <v>00:44:02</v>
       </c>
     </row>
     <row r="7">
@@ -1317,13 +1062,13 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D7" t="str">
-        <v>00:30:43</v>
+        <v>02:06:57</v>
       </c>
     </row>
     <row r="8">
@@ -1331,172 +1076,102 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D8" t="str">
-        <v>02:48:34</v>
+        <v>02:20:22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-16</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" t="str">
-        <v>01:30:45</v>
+        <v>00:12:38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-16</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" t="str">
-        <v>02:28:48</v>
+        <v>00:04:44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MAXUS SRYB-26 (NOVA-ANF)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-13</v>
       </c>
       <c r="C11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" t="str">
-        <v>00:57:06</v>
+        <v>01:50:23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="str">
-        <v>00:01:39</v>
+        <v>00:49:34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-16</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>00:02:54</v>
+        <v>01:29:10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>PEUGEOT SVCH-53 (STGO)</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="str">
-        <v>00:16:39</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
-      </c>
-      <c r="B15" t="str">
-        <v>2026-10-08</v>
-      </c>
-      <c r="C15">
-        <v>4</v>
-      </c>
-      <c r="D15" t="str">
-        <v>01:17:32</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
-      </c>
-      <c r="B16" t="str">
-        <v>2026-10-05</v>
-      </c>
-      <c r="C16">
-        <v>4</v>
-      </c>
-      <c r="D16" t="str">
-        <v>00:20:49</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B17" t="str">
-        <v>2026-10-07</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" t="str">
-        <v>00:04:06</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>MITSUBISHI VDYY-73 (Chillan)</v>
-      </c>
-      <c r="B18" t="str">
-        <v>2026-10-09</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18" t="str">
-        <v>00:29:28</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>PEUGEOT SVCH-53 (STGO)</v>
-      </c>
-      <c r="B19" t="str">
-        <v>2026-10-07</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" t="str">
-        <v>00:09:05</v>
+        <v>00:07:57</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1518,35 +1193,35 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FORD VYVC-51 (TALLER-ANF)</v>
+        <v>FORD RANGER VYVC-38 (STGO PR)</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>00:52:05</v>
+        <v>01:16:42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FORD VYVC-65 (TALLER-ANF)</v>
+        <v>FORD VYVC-51 (TALLER-ANF)</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>00:02:14</v>
+        <v>00:06:09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>L200 VDYY-82 (CENIZA-ANF)</v>
+        <v>FORD VYVC-65 (TALLER-ANF)</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="str">
-        <v>00:13:01</v>
+        <v>00:04:54</v>
       </c>
     </row>
     <row r="5">
@@ -1554,43 +1229,43 @@
         <v>MAXUS SRYB-26 (NOVA-ANF)</v>
       </c>
       <c r="B5">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>08:15:56</v>
+        <v>05:11:21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MAXUS TVVB-25 (CHILLAN)</v>
+        <v>MAXUS TFWK-88 (STGO)</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="str">
-        <v>00:01:39</v>
+        <v>00:12:38</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
+        <v>MAXUS TVVB-26 (STGO)</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>01:37:05</v>
+        <v>00:04:44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MAXUS VGVV-79 (STGO MA)</v>
+        <v>MAXUS TYTC-88 (NOVA-ANF)</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="str">
-        <v>00:20:49</v>
+        <v>01:50:23</v>
       </c>
     </row>
     <row r="9">
@@ -1598,10 +1273,10 @@
         <v>MITSUBISHI VDYY-73 (Chillan)</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C9" t="str">
-        <v>00:33:34</v>
+        <v>02:18:44</v>
       </c>
     </row>
     <row r="10">
@@ -1612,7 +1287,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="str">
-        <v>00:09:05</v>
+        <v>00:07:57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>